<commit_message>
feat: dong bo toan dien web, bao cao, HDSD va toi uu 5 day xien & de neo dung chung
</commit_message>
<xml_diff>
--- a/docs/mat-bang-neo-9-be/bang_thong_ke_neo_9_be.xlsx
+++ b/docs/mat-bang-neo-9-be/bang_thong_ke_neo_9_be.xlsx
@@ -3184,13 +3184,13 @@
         <v>BÈ 3</v>
       </c>
       <c r="D49">
-        <v>-41.3</v>
+        <v>-35.8</v>
       </c>
       <c r="E49">
-        <v>-149.57</v>
+        <v>-179.26</v>
       </c>
       <c r="F49">
-        <v>384.08</v>
+        <v>385.08</v>
       </c>
       <c r="G49">
         <v>1</v>
@@ -7462,13 +7462,13 @@
         <v>BÈ 5A</v>
       </c>
       <c r="D118">
-        <v>419.48</v>
+        <v>423.01</v>
       </c>
       <c r="E118">
-        <v>-154.12</v>
+        <v>-168.16</v>
       </c>
       <c r="F118">
-        <v>384.2</v>
+        <v>388.57</v>
       </c>
       <c r="G118">
         <v>1</v>
@@ -7524,13 +7524,13 @@
         <v>BÈ 5A</v>
       </c>
       <c r="D119">
-        <v>420.28</v>
+        <v>418.19</v>
       </c>
       <c r="E119">
-        <v>-149.28</v>
+        <v>-162.96</v>
       </c>
       <c r="F119">
-        <v>384.75</v>
+        <v>384</v>
       </c>
       <c r="G119">
         <v>1</v>
@@ -10748,13 +10748,13 @@
         <v>BÈ 7</v>
       </c>
       <c r="D171">
-        <v>76.46</v>
+        <v>81.73</v>
       </c>
       <c r="E171">
-        <v>-76.01</v>
+        <v>-97.29</v>
       </c>
       <c r="F171">
-        <v>384.07</v>
+        <v>384.1</v>
       </c>
       <c r="G171">
         <v>1</v>
@@ -12484,13 +12484,13 @@
         <v>BÈ 8</v>
       </c>
       <c r="D199">
-        <v>41.03</v>
+        <v>47.33</v>
       </c>
       <c r="E199">
-        <v>92.56</v>
+        <v>71.85</v>
       </c>
       <c r="F199">
-        <v>384.03</v>
+        <v>384.01</v>
       </c>
       <c r="G199">
         <v>1</v>
@@ -15048,19 +15048,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E7">
-        <v>-139.37</v>
+        <v>-138.58</v>
       </c>
       <c r="F7">
-        <v>30.03</v>
+        <v>31.21</v>
       </c>
       <c r="G7">
         <v>378.3</v>
       </c>
       <c r="H7">
-        <v>11.07</v>
+        <v>11.3</v>
       </c>
       <c r="I7">
-        <v>143.4</v>
+        <v>136.6</v>
       </c>
       <c r="J7">
         <v>2.5</v>
@@ -15090,10 +15090,10 @@
         <v>0.47</v>
       </c>
       <c r="S7">
-        <v>0.28</v>
+        <v>0.27</v>
       </c>
       <c r="T7">
-        <v>0.5</v>
+        <v>0.47</v>
       </c>
       <c r="U7">
         <v>0</v>
@@ -15196,19 +15196,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E9">
-        <v>-48.11</v>
+        <v>-48.54</v>
       </c>
       <c r="F9">
-        <v>-33.37</v>
+        <v>-35.03</v>
       </c>
       <c r="G9">
         <v>378.3</v>
       </c>
       <c r="H9">
-        <v>8.91</v>
+        <v>9.01</v>
       </c>
       <c r="I9">
-        <v>102.6</v>
+        <v>113.6</v>
       </c>
       <c r="J9">
         <v>2.5</v>
@@ -15235,16 +15235,16 @@
         <v>38.6</v>
       </c>
       <c r="R9">
-        <v>0.62</v>
+        <v>0.63</v>
       </c>
       <c r="S9">
-        <v>0.37</v>
+        <v>0.36</v>
       </c>
       <c r="T9">
-        <v>0.69</v>
+        <v>0.67</v>
       </c>
       <c r="U9">
-        <v>0.43</v>
+        <v>0.38</v>
       </c>
       <c r="V9">
         <v>0.15</v>
@@ -15270,19 +15270,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E10">
-        <v>-25.86</v>
+        <v>-28.46</v>
       </c>
       <c r="F10">
-        <v>-15.46</v>
+        <v>-18.93</v>
       </c>
       <c r="G10">
         <v>378.3</v>
       </c>
       <c r="H10">
-        <v>13.98</v>
+        <v>14.23</v>
       </c>
       <c r="I10">
-        <v>121.3</v>
+        <v>138.9</v>
       </c>
       <c r="J10">
         <v>2.5</v>
@@ -15309,16 +15309,16 @@
         <v>38.6</v>
       </c>
       <c r="R10">
-        <v>0.44</v>
+        <v>0.46</v>
       </c>
       <c r="S10">
-        <v>0.38</v>
+        <v>0.37</v>
       </c>
       <c r="T10">
-        <v>0.56</v>
+        <v>0.51</v>
       </c>
       <c r="U10">
-        <v>0.12</v>
+        <v>0.01</v>
       </c>
       <c r="V10">
         <v>0.15</v>
@@ -15344,19 +15344,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E11">
-        <v>18.01</v>
+        <v>16.6</v>
       </c>
       <c r="F11">
-        <v>-122.77</v>
+        <v>-124.06</v>
       </c>
       <c r="G11">
         <v>378.3</v>
       </c>
       <c r="H11">
-        <v>9.54</v>
+        <v>9.35</v>
       </c>
       <c r="I11">
-        <v>126.5</v>
+        <v>138</v>
       </c>
       <c r="J11">
         <v>3.25</v>
@@ -15383,16 +15383,16 @@
         <v>73.7</v>
       </c>
       <c r="R11">
-        <v>0.76</v>
+        <v>0.77</v>
       </c>
       <c r="S11">
-        <v>0.62</v>
+        <v>0.55</v>
       </c>
       <c r="T11">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="U11">
-        <v>0.71</v>
+        <v>0.68</v>
       </c>
       <c r="V11">
         <v>0.15</v>
@@ -15418,34 +15418,34 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E12">
-        <v>49.15</v>
+        <v>42.39</v>
       </c>
       <c r="F12">
-        <v>-116.18</v>
+        <v>-119.37</v>
       </c>
       <c r="G12">
         <v>378.3</v>
       </c>
       <c r="H12">
-        <v>15.18</v>
+        <v>15.33</v>
       </c>
       <c r="I12">
-        <v>116.8</v>
+        <v>139.5</v>
       </c>
       <c r="J12">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="K12">
         <v>0.4</v>
       </c>
       <c r="L12">
-        <v>3.01</v>
+        <v>2.48</v>
       </c>
       <c r="M12">
-        <v>141</v>
+        <v>119</v>
       </c>
       <c r="N12">
-        <v>7.7</v>
+        <v>6.4</v>
       </c>
       <c r="O12">
         <v>4</v>
@@ -15457,16 +15457,16 @@
         <v>73.7</v>
       </c>
       <c r="R12">
-        <v>0.62</v>
+        <v>0.73</v>
       </c>
       <c r="S12">
-        <v>0.69</v>
+        <v>0.75</v>
       </c>
       <c r="T12">
         <v>0.91</v>
       </c>
       <c r="U12">
-        <v>0.84</v>
+        <v>0.93</v>
       </c>
       <c r="V12">
         <v>0.15</v>
@@ -15492,34 +15492,34 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E13">
-        <v>33.69</v>
+        <v>29.5</v>
       </c>
       <c r="F13">
-        <v>-119.71</v>
+        <v>-121.71</v>
       </c>
       <c r="G13">
         <v>378.3</v>
       </c>
       <c r="H13">
-        <v>11.97</v>
+        <v>12.34</v>
       </c>
       <c r="I13">
-        <v>120.7</v>
+        <v>138.9</v>
       </c>
       <c r="J13">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="K13">
         <v>0.4</v>
       </c>
       <c r="L13">
-        <v>3.58</v>
+        <v>3.01</v>
       </c>
       <c r="M13">
-        <v>165</v>
+        <v>141</v>
       </c>
       <c r="N13">
-        <v>9.2</v>
+        <v>7.7</v>
       </c>
       <c r="O13">
         <v>4</v>
@@ -15531,16 +15531,16 @@
         <v>73.7</v>
       </c>
       <c r="R13">
-        <v>0.69</v>
+        <v>0.78</v>
       </c>
       <c r="S13">
-        <v>0.83</v>
+        <v>0.67</v>
       </c>
       <c r="T13">
-        <v>0.91</v>
+        <v>0.94</v>
       </c>
       <c r="U13">
-        <v>0.74</v>
+        <v>0.92</v>
       </c>
       <c r="V13">
         <v>0.15</v>
@@ -15566,34 +15566,34 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E14">
-        <v>0.59</v>
+        <v>5.97</v>
       </c>
       <c r="F14">
-        <v>-131.46</v>
+        <v>-128.68</v>
       </c>
       <c r="G14">
         <v>378.3</v>
       </c>
       <c r="H14">
-        <v>9.76</v>
+        <v>9.59</v>
       </c>
       <c r="I14">
-        <v>172.3</v>
+        <v>135.9</v>
       </c>
       <c r="J14">
-        <v>3.25</v>
+        <v>3</v>
       </c>
       <c r="K14">
         <v>0.4</v>
       </c>
       <c r="L14">
-        <v>4.21</v>
+        <v>3.58</v>
       </c>
       <c r="M14">
-        <v>202</v>
+        <v>165</v>
       </c>
       <c r="N14">
-        <v>10.8</v>
+        <v>9.2</v>
       </c>
       <c r="O14">
         <v>4</v>
@@ -15605,16 +15605,16 @@
         <v>73.7</v>
       </c>
       <c r="R14">
-        <v>0.66</v>
+        <v>0.84</v>
       </c>
       <c r="S14">
-        <v>0.58</v>
+        <v>0.61</v>
       </c>
       <c r="T14">
-        <v>0.93</v>
+        <v>0.99</v>
       </c>
       <c r="U14">
-        <v>0.71</v>
+        <v>0.96</v>
       </c>
       <c r="V14">
         <v>0.15</v>
@@ -16380,19 +16380,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E25">
-        <v>172.09</v>
+        <v>170.95</v>
       </c>
       <c r="F25">
-        <v>-80.6</v>
+        <v>-78.93</v>
       </c>
       <c r="G25">
         <v>378.3</v>
       </c>
       <c r="H25">
-        <v>12.97</v>
+        <v>14.34</v>
       </c>
       <c r="I25">
-        <v>16.4</v>
+        <v>10.2</v>
       </c>
       <c r="J25">
         <v>2.75</v>
@@ -16419,16 +16419,16 @@
         <v>73.7</v>
       </c>
       <c r="R25">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
       <c r="S25">
         <v>0.67</v>
       </c>
       <c r="T25">
-        <v>0.89</v>
+        <v>0.87</v>
       </c>
       <c r="U25">
-        <v>0.79</v>
+        <v>0.75</v>
       </c>
       <c r="V25">
         <v>0.15</v>
@@ -16454,19 +16454,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E26">
-        <v>157.75</v>
+        <v>156.82</v>
       </c>
       <c r="F26">
-        <v>-78.99</v>
+        <v>-78.93</v>
       </c>
       <c r="G26">
         <v>378.3</v>
       </c>
       <c r="H26">
-        <v>14.29</v>
+        <v>14.36</v>
       </c>
       <c r="I26">
-        <v>14.3</v>
+        <v>10.6</v>
       </c>
       <c r="J26">
         <v>2.75</v>
@@ -16499,7 +16499,7 @@
         <v>0.67</v>
       </c>
       <c r="T26">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="U26">
         <v>0.75</v>
@@ -16528,19 +16528,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E27">
-        <v>143.31</v>
+        <v>142.07</v>
       </c>
       <c r="F27">
-        <v>-78.94</v>
+        <v>-78.93</v>
       </c>
       <c r="G27">
         <v>378.3</v>
       </c>
       <c r="H27">
-        <v>14.18</v>
+        <v>14.31</v>
       </c>
       <c r="I27">
-        <v>14.5</v>
+        <v>9.7</v>
       </c>
       <c r="J27">
         <v>2.75</v>
@@ -16570,13 +16570,13 @@
         <v>0.73</v>
       </c>
       <c r="S27">
-        <v>0.68</v>
+        <v>0.67</v>
       </c>
       <c r="T27">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="U27">
-        <v>0.77</v>
+        <v>0.75</v>
       </c>
       <c r="V27">
         <v>0.15</v>
@@ -16602,19 +16602,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E28">
-        <v>128.93</v>
+        <v>127.95</v>
       </c>
       <c r="F28">
-        <v>-79.36</v>
+        <v>-78.93</v>
       </c>
       <c r="G28">
         <v>378.3</v>
       </c>
       <c r="H28">
-        <v>14.12</v>
+        <v>14.34</v>
       </c>
       <c r="I28">
-        <v>14.4</v>
+        <v>10.2</v>
       </c>
       <c r="J28">
         <v>2.75</v>
@@ -16647,10 +16647,10 @@
         <v>0.67</v>
       </c>
       <c r="T28">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="U28">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="V28">
         <v>0.15</v>
@@ -16676,19 +16676,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E29">
-        <v>114.44</v>
+        <v>113.2</v>
       </c>
       <c r="F29">
-        <v>-78.94</v>
+        <v>-78.93</v>
       </c>
       <c r="G29">
         <v>378.3</v>
       </c>
       <c r="H29">
-        <v>14.17</v>
+        <v>14.29</v>
       </c>
       <c r="I29">
-        <v>14</v>
+        <v>9.2</v>
       </c>
       <c r="J29">
         <v>2.75</v>
@@ -16715,16 +16715,16 @@
         <v>73.7</v>
       </c>
       <c r="R29">
-        <v>0.73</v>
+        <v>0.74</v>
       </c>
       <c r="S29">
-        <v>0.68</v>
+        <v>0.67</v>
       </c>
       <c r="T29">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="U29">
-        <v>0.77</v>
+        <v>0.75</v>
       </c>
       <c r="V29">
         <v>0.15</v>
@@ -16750,34 +16750,34 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E30">
-        <v>371.71</v>
+        <v>369.3</v>
       </c>
       <c r="F30">
-        <v>-73.49</v>
+        <v>-73.82</v>
       </c>
       <c r="G30">
         <v>378.3</v>
       </c>
       <c r="H30">
-        <v>20.76</v>
+        <v>21.3</v>
       </c>
       <c r="I30">
-        <v>14.4</v>
+        <v>8.3</v>
       </c>
       <c r="J30">
-        <v>2.5</v>
+        <v>2.75</v>
       </c>
       <c r="K30">
         <v>0.4</v>
       </c>
       <c r="L30">
-        <v>2.48</v>
+        <v>3.01</v>
       </c>
       <c r="M30">
-        <v>119</v>
+        <v>141</v>
       </c>
       <c r="N30">
-        <v>6.4</v>
+        <v>7.7</v>
       </c>
       <c r="O30">
         <v>4</v>
@@ -16789,16 +16789,16 @@
         <v>87.3</v>
       </c>
       <c r="R30">
-        <v>0.61</v>
+        <v>0.56</v>
       </c>
       <c r="S30">
-        <v>0.92</v>
+        <v>0.81</v>
       </c>
       <c r="T30">
-        <v>0.94</v>
+        <v>0.84</v>
       </c>
       <c r="U30">
-        <v>0.98</v>
+        <v>0.66</v>
       </c>
       <c r="V30">
         <v>0.15</v>
@@ -16898,19 +16898,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E32">
-        <v>337.83</v>
+        <v>346.24</v>
       </c>
       <c r="F32">
-        <v>-69.35</v>
+        <v>-75.68</v>
       </c>
       <c r="G32">
         <v>378.3</v>
       </c>
       <c r="H32">
-        <v>22.08</v>
+        <v>21.45</v>
       </c>
       <c r="I32">
-        <v>2.5</v>
+        <v>26.3</v>
       </c>
       <c r="J32">
         <v>2.75</v>
@@ -16937,16 +16937,16 @@
         <v>87.3</v>
       </c>
       <c r="R32">
-        <v>0.5</v>
+        <v>0.56</v>
       </c>
       <c r="S32">
+        <v>0.81</v>
+      </c>
+      <c r="T32">
         <v>0.83</v>
       </c>
-      <c r="T32">
-        <v>0.87</v>
-      </c>
       <c r="U32">
-        <v>0.74</v>
+        <v>0.65</v>
       </c>
       <c r="V32">
         <v>0.15</v>
@@ -16972,19 +16972,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E33">
-        <v>111.96</v>
+        <v>110.63</v>
       </c>
       <c r="F33">
-        <v>89.82</v>
+        <v>90.49</v>
       </c>
       <c r="G33">
         <v>378.3</v>
       </c>
       <c r="H33">
-        <v>10.67</v>
+        <v>11.52</v>
       </c>
       <c r="I33">
-        <v>355.2</v>
+        <v>348.9</v>
       </c>
       <c r="J33">
         <v>2.5</v>
@@ -17017,10 +17017,10 @@
         <v>0.59</v>
       </c>
       <c r="T33">
-        <v>0.92</v>
+        <v>0.9</v>
       </c>
       <c r="U33">
-        <v>0.95</v>
+        <v>0.89</v>
       </c>
       <c r="V33">
         <v>0.15</v>
@@ -17049,16 +17049,16 @@
         <v>130.63</v>
       </c>
       <c r="F34">
-        <v>93.62</v>
+        <v>90.49</v>
       </c>
       <c r="G34">
         <v>378.3</v>
       </c>
       <c r="H34">
-        <v>11.6</v>
+        <v>13.97</v>
       </c>
       <c r="I34">
-        <v>330.3</v>
+        <v>324</v>
       </c>
       <c r="J34">
         <v>2.5</v>
@@ -17085,16 +17085,16 @@
         <v>59.1</v>
       </c>
       <c r="R34">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
       <c r="S34">
         <v>0.59</v>
       </c>
       <c r="T34">
-        <v>0.83</v>
+        <v>0.79</v>
       </c>
       <c r="U34">
-        <v>0.74</v>
+        <v>0.65</v>
       </c>
       <c r="V34">
         <v>0.15</v>
@@ -17123,16 +17123,16 @@
         <v>83.63</v>
       </c>
       <c r="F35">
-        <v>87.37</v>
+        <v>90.49</v>
       </c>
       <c r="G35">
         <v>378.3</v>
       </c>
       <c r="H35">
-        <v>8.79</v>
+        <v>11.75</v>
       </c>
       <c r="I35">
-        <v>338.5</v>
+        <v>344.1</v>
       </c>
       <c r="J35">
         <v>2.5</v>
@@ -17165,10 +17165,10 @@
         <v>0.59</v>
       </c>
       <c r="T35">
-        <v>0.94</v>
+        <v>0.89</v>
       </c>
       <c r="U35">
-        <v>0.98</v>
+        <v>0.87</v>
       </c>
       <c r="V35">
         <v>0.15</v>
@@ -17268,19 +17268,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E37">
-        <v>115.24</v>
+        <v>121.79</v>
       </c>
       <c r="F37">
-        <v>293.32</v>
+        <v>292.95</v>
       </c>
       <c r="G37">
         <v>378.3</v>
       </c>
       <c r="H37">
-        <v>12.14</v>
+        <v>11.49</v>
       </c>
       <c r="I37">
-        <v>341.8</v>
+        <v>13.8</v>
       </c>
       <c r="J37">
         <v>2.5</v>
@@ -17307,16 +17307,16 @@
         <v>59.1</v>
       </c>
       <c r="R37">
-        <v>0.67</v>
+        <v>0.73</v>
       </c>
       <c r="S37">
-        <v>0.87</v>
+        <v>0.59</v>
       </c>
       <c r="T37">
-        <v>0.94</v>
+        <v>0.86</v>
       </c>
       <c r="U37">
-        <v>0.98</v>
+        <v>0.82</v>
       </c>
       <c r="V37">
         <v>0.15</v>
@@ -17376,7 +17376,7 @@
         <v>Tổng bê tông đế</v>
       </c>
       <c r="B43">
-        <v>93.4</v>
+        <v>92.2</v>
       </c>
       <c r="C43" t="str">
         <v>m³</v>
@@ -17387,7 +17387,7 @@
         <v>Tổng thép bản đế (ước tính)</v>
       </c>
       <c r="B44">
-        <v>4.42</v>
+        <v>4.36</v>
       </c>
       <c r="C44" t="str">
         <v>tấn</v>
@@ -17561,19 +17561,19 @@
         <v>Ø12 a200</v>
       </c>
       <c r="F4">
-        <v>4.6</v>
+        <v>4.8</v>
       </c>
       <c r="G4">
-        <v>28.9</v>
+        <v>29.7</v>
       </c>
       <c r="H4">
         <v>30.1</v>
       </c>
       <c r="I4">
-        <v>14.6</v>
+        <v>15</v>
       </c>
       <c r="J4">
-        <v>0.22</v>
+        <v>0.23</v>
       </c>
       <c r="K4">
         <v>0.33</v>
@@ -17614,16 +17614,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="F5">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="G5">
-        <v>36.8</v>
+        <v>36.5</v>
       </c>
       <c r="H5">
         <v>27.6</v>
       </c>
       <c r="I5">
-        <v>16.6</v>
+        <v>16.5</v>
       </c>
       <c r="J5">
         <v>0.25</v>
@@ -17667,19 +17667,19 @@
         <v>Ø12 a200</v>
       </c>
       <c r="F6">
-        <v>5.8</v>
+        <v>6</v>
       </c>
       <c r="G6">
-        <v>35.3</v>
+        <v>36.5</v>
       </c>
       <c r="H6">
         <v>38.4</v>
       </c>
       <c r="I6">
-        <v>22.3</v>
+        <v>23</v>
       </c>
       <c r="J6">
-        <v>0.34</v>
+        <v>0.35</v>
       </c>
       <c r="K6">
         <v>0.42</v>
@@ -17688,7 +17688,7 @@
         <v>0.54</v>
       </c>
       <c r="M6">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="N6">
         <v>0.15</v>
@@ -17720,19 +17720,19 @@
         <v>Ø12 a200</v>
       </c>
       <c r="F7">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="G7">
-        <v>35</v>
+        <v>35.6</v>
       </c>
       <c r="H7">
         <v>73.3</v>
       </c>
       <c r="I7">
-        <v>42.2</v>
+        <v>42.8</v>
       </c>
       <c r="J7">
-        <v>0.58</v>
+        <v>0.59</v>
       </c>
       <c r="K7">
         <v>0.72</v>
@@ -17741,7 +17741,7 @@
         <v>0.92</v>
       </c>
       <c r="M7">
-        <v>0.85</v>
+        <v>0.87</v>
       </c>
       <c r="N7">
         <v>0.15</v>
@@ -17826,28 +17826,28 @@
         <v>Ø12 a200</v>
       </c>
       <c r="F9">
-        <v>6.2</v>
+        <v>4.8</v>
       </c>
       <c r="G9">
-        <v>37.4</v>
+        <v>30.5</v>
       </c>
       <c r="H9">
-        <v>45.3</v>
+        <v>45.4</v>
       </c>
       <c r="I9">
-        <v>27.7</v>
+        <v>23.1</v>
       </c>
       <c r="J9">
-        <v>0.42</v>
+        <v>0.35</v>
       </c>
       <c r="K9">
-        <v>0.49</v>
+        <v>0.5</v>
       </c>
       <c r="L9">
-        <v>0.65</v>
+        <v>0.6</v>
       </c>
       <c r="M9">
-        <v>0.33</v>
+        <v>0.22</v>
       </c>
       <c r="N9">
         <v>0.15</v>
@@ -17985,25 +17985,25 @@
         <v>Ø12 a200</v>
       </c>
       <c r="F12">
-        <v>3.8</v>
+        <v>4.8</v>
       </c>
       <c r="G12">
-        <v>25.1</v>
+        <v>30.3</v>
       </c>
       <c r="H12">
         <v>30.8</v>
       </c>
       <c r="I12">
-        <v>13.1</v>
+        <v>15.6</v>
       </c>
       <c r="J12">
-        <v>0.2</v>
+        <v>0.24</v>
       </c>
       <c r="K12">
         <v>0.34</v>
       </c>
       <c r="L12">
-        <v>0.38</v>
+        <v>0.41</v>
       </c>
       <c r="M12">
         <v>0</v>
@@ -18328,7 +18328,7 @@
         <v>30.2</v>
       </c>
       <c r="G8">
-        <v>11.7</v>
+        <v>11.3</v>
       </c>
       <c r="H8" t="str">
         <v>B2-D20</v>
@@ -18340,19 +18340,19 @@
         <v>27.8</v>
       </c>
       <c r="K8">
-        <v>11.07</v>
+        <v>11.3</v>
       </c>
       <c r="L8">
-        <v>-139.37</v>
+        <v>-138.58</v>
       </c>
       <c r="M8">
-        <v>30.03</v>
+        <v>31.21</v>
       </c>
       <c r="N8">
         <v>378.3</v>
       </c>
       <c r="O8">
-        <v>378.87</v>
+        <v>378.71</v>
       </c>
       <c r="P8">
         <v>1.7</v>
@@ -18364,10 +18364,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S8">
-        <v>6.4</v>
+        <v>2.1</v>
       </c>
       <c r="T8">
-        <v>30.8</v>
+        <v>31</v>
       </c>
       <c r="U8">
         <v>2.5</v>
@@ -18391,10 +18391,10 @@
         <v>0.47</v>
       </c>
       <c r="AB8">
-        <v>0.28</v>
+        <v>0.27</v>
       </c>
       <c r="AC8">
-        <v>0.5</v>
+        <v>0.47</v>
       </c>
       <c r="AD8">
         <v>0</v>
@@ -18412,7 +18412,7 @@
         <v>ĐẠT</v>
       </c>
       <c r="AI8" t="str">
-        <v>Đế dùng chung hai bè: hai tai neo; Địa hình IFC tại điểm này cao hơn đáy thiết kế 0,6 m: kiểm tra khảo sát / nạo vét trước khi đặt đế</v>
+        <v>Đế dùng chung hai bè: hai tai neo</v>
       </c>
     </row>
     <row r="9">
@@ -18542,7 +18542,7 @@
         <v>27.8</v>
       </c>
       <c r="G10">
-        <v>8.91</v>
+        <v>9.01</v>
       </c>
       <c r="H10" t="str">
         <v>B3-D17</v>
@@ -18554,13 +18554,13 @@
         <v>38.6</v>
       </c>
       <c r="K10">
-        <v>9.44</v>
+        <v>9.02</v>
       </c>
       <c r="L10">
-        <v>-48.11</v>
+        <v>-48.54</v>
       </c>
       <c r="M10">
-        <v>-33.37</v>
+        <v>-35.03</v>
       </c>
       <c r="N10">
         <v>378.3</v>
@@ -18578,10 +18578,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S10">
-        <v>13.3</v>
+        <v>8.5</v>
       </c>
       <c r="T10">
-        <v>40.7</v>
+        <v>41.3</v>
       </c>
       <c r="U10">
         <v>2.5</v>
@@ -18602,16 +18602,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA10">
-        <v>0.62</v>
+        <v>0.63</v>
       </c>
       <c r="AB10">
-        <v>0.37</v>
+        <v>0.36</v>
       </c>
       <c r="AC10">
-        <v>0.69</v>
+        <v>0.67</v>
       </c>
       <c r="AD10">
-        <v>0.43</v>
+        <v>0.38</v>
       </c>
       <c r="AE10">
         <v>0.15</v>
@@ -18620,7 +18620,7 @@
         <v>0.62</v>
       </c>
       <c r="AG10">
-        <v>0.69</v>
+        <v>0.67</v>
       </c>
       <c r="AH10" t="str">
         <v>ĐẠT</v>
@@ -18649,7 +18649,7 @@
         <v>27.8</v>
       </c>
       <c r="G11">
-        <v>13.98</v>
+        <v>14.23</v>
       </c>
       <c r="H11" t="str">
         <v>B3-D13</v>
@@ -18661,19 +18661,19 @@
         <v>38.6</v>
       </c>
       <c r="K11">
-        <v>15.72</v>
+        <v>14.23</v>
       </c>
       <c r="L11">
-        <v>-25.86</v>
+        <v>-28.46</v>
       </c>
       <c r="M11">
-        <v>-15.46</v>
+        <v>-18.93</v>
       </c>
       <c r="N11">
         <v>378.3</v>
       </c>
       <c r="O11">
-        <v>378.54</v>
+        <v>378.5</v>
       </c>
       <c r="P11">
         <v>1.7</v>
@@ -18685,10 +18685,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S11">
-        <v>19.9</v>
+        <v>9.7</v>
       </c>
       <c r="T11">
-        <v>28.6</v>
+        <v>29.8</v>
       </c>
       <c r="U11">
         <v>2.5</v>
@@ -18709,16 +18709,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA11">
-        <v>0.44</v>
+        <v>0.46</v>
       </c>
       <c r="AB11">
-        <v>0.38</v>
+        <v>0.37</v>
       </c>
       <c r="AC11">
-        <v>0.56</v>
+        <v>0.51</v>
       </c>
       <c r="AD11">
-        <v>0.12</v>
+        <v>0.01</v>
       </c>
       <c r="AE11">
         <v>0.15</v>
@@ -18756,7 +18756,7 @@
         <v>38.6</v>
       </c>
       <c r="G12">
-        <v>9.54</v>
+        <v>9.36</v>
       </c>
       <c r="H12" t="str">
         <v>B3A-D23</v>
@@ -18768,13 +18768,13 @@
         <v>73.7</v>
       </c>
       <c r="K12">
-        <v>9.56</v>
+        <v>9.35</v>
       </c>
       <c r="L12">
-        <v>18.01</v>
+        <v>16.6</v>
       </c>
       <c r="M12">
-        <v>-122.77</v>
+        <v>-124.06</v>
       </c>
       <c r="N12">
         <v>378.3</v>
@@ -18792,10 +18792,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S12">
-        <v>32.9</v>
+        <v>27.8</v>
       </c>
       <c r="T12">
-        <v>67.3</v>
+        <v>68.2</v>
       </c>
       <c r="U12">
         <v>3.25</v>
@@ -18816,16 +18816,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA12">
-        <v>0.76</v>
+        <v>0.77</v>
       </c>
       <c r="AB12">
-        <v>0.62</v>
+        <v>0.55</v>
       </c>
       <c r="AC12">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="AD12">
-        <v>0.71</v>
+        <v>0.68</v>
       </c>
       <c r="AE12">
         <v>0.15</v>
@@ -18834,7 +18834,7 @@
         <v>0.62</v>
       </c>
       <c r="AG12">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="AH12" t="str">
         <v>ĐẠT</v>
@@ -18863,7 +18863,7 @@
         <v>38.6</v>
       </c>
       <c r="G13">
-        <v>18.74</v>
+        <v>15.33</v>
       </c>
       <c r="H13" t="str">
         <v>B3A-D21</v>
@@ -18875,19 +18875,19 @@
         <v>73.7</v>
       </c>
       <c r="K13">
-        <v>15.18</v>
+        <v>15.33</v>
       </c>
       <c r="L13">
-        <v>49.15</v>
+        <v>42.39</v>
       </c>
       <c r="M13">
-        <v>-116.18</v>
+        <v>-119.37</v>
       </c>
       <c r="N13">
         <v>378.3</v>
       </c>
       <c r="O13">
-        <v>378.89</v>
+        <v>378.5</v>
       </c>
       <c r="P13">
         <v>1.7</v>
@@ -18899,40 +18899,40 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S13">
-        <v>52.1</v>
+        <v>31.7</v>
       </c>
       <c r="T13">
-        <v>45.2</v>
+        <v>47.5</v>
       </c>
       <c r="U13">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="V13">
         <v>0.4</v>
       </c>
       <c r="W13">
-        <v>45.4</v>
+        <v>37.5</v>
       </c>
       <c r="X13">
-        <v>3.01</v>
+        <v>2.48</v>
       </c>
       <c r="Y13">
-        <v>7.7</v>
+        <v>6.4</v>
       </c>
       <c r="Z13" t="str">
         <v>Ø12 a200</v>
       </c>
       <c r="AA13">
-        <v>0.62</v>
+        <v>0.73</v>
       </c>
       <c r="AB13">
-        <v>0.69</v>
+        <v>0.75</v>
       </c>
       <c r="AC13">
         <v>0.91</v>
       </c>
       <c r="AD13">
-        <v>0.84</v>
+        <v>0.93</v>
       </c>
       <c r="AE13">
         <v>0.15</v>
@@ -18941,13 +18941,13 @@
         <v>0.62</v>
       </c>
       <c r="AG13">
-        <v>0.91</v>
+        <v>0.93</v>
       </c>
       <c r="AH13" t="str">
         <v>ĐẠT</v>
       </c>
       <c r="AI13" t="str">
-        <v>Đế dùng chung hai bè: hai tai neo; Địa hình IFC tại điểm này cao hơn đáy thiết kế 0,6 m: kiểm tra khảo sát / nạo vét trước khi đặt đế; Đế lớn hơn đế mẫu</v>
+        <v>Đế dùng chung hai bè: hai tai neo</v>
       </c>
     </row>
     <row r="14">
@@ -18970,7 +18970,7 @@
         <v>38.6</v>
       </c>
       <c r="G14">
-        <v>14.3</v>
+        <v>12.34</v>
       </c>
       <c r="H14" t="str">
         <v>B3A-D22</v>
@@ -18982,13 +18982,13 @@
         <v>73.7</v>
       </c>
       <c r="K14">
-        <v>11.97</v>
+        <v>12.34</v>
       </c>
       <c r="L14">
-        <v>33.69</v>
+        <v>29.5</v>
       </c>
       <c r="M14">
-        <v>-119.71</v>
+        <v>-121.71</v>
       </c>
       <c r="N14">
         <v>378.3</v>
@@ -19006,40 +19006,40 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S14">
-        <v>43.1</v>
+        <v>30.3</v>
       </c>
       <c r="T14">
-        <v>55.1</v>
+        <v>56.3</v>
       </c>
       <c r="U14">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="V14">
         <v>0.4</v>
       </c>
       <c r="W14">
-        <v>54</v>
+        <v>45.4</v>
       </c>
       <c r="X14">
-        <v>3.58</v>
+        <v>3.01</v>
       </c>
       <c r="Y14">
-        <v>9.2</v>
+        <v>7.7</v>
       </c>
       <c r="Z14" t="str">
         <v>Ø12 a200</v>
       </c>
       <c r="AA14">
-        <v>0.69</v>
+        <v>0.78</v>
       </c>
       <c r="AB14">
-        <v>0.83</v>
+        <v>0.67</v>
       </c>
       <c r="AC14">
-        <v>0.91</v>
+        <v>0.94</v>
       </c>
       <c r="AD14">
-        <v>0.74</v>
+        <v>0.92</v>
       </c>
       <c r="AE14">
         <v>0.15</v>
@@ -19048,7 +19048,7 @@
         <v>0.62</v>
       </c>
       <c r="AG14">
-        <v>0.91</v>
+        <v>0.94</v>
       </c>
       <c r="AH14" t="str">
         <v>ĐẠT</v>
@@ -19077,7 +19077,7 @@
         <v>38.6</v>
       </c>
       <c r="G15">
-        <v>9.76</v>
+        <v>9.6</v>
       </c>
       <c r="H15" t="str">
         <v>B3A-D24</v>
@@ -19089,13 +19089,13 @@
         <v>73.7</v>
       </c>
       <c r="K15">
-        <v>12.73</v>
+        <v>9.59</v>
       </c>
       <c r="L15">
-        <v>0.59</v>
+        <v>5.97</v>
       </c>
       <c r="M15">
-        <v>-131.46</v>
+        <v>-128.68</v>
       </c>
       <c r="N15">
         <v>378.3</v>
@@ -19113,40 +19113,40 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S15">
-        <v>57.5</v>
+        <v>28.1</v>
       </c>
       <c r="T15">
-        <v>58.9</v>
+        <v>67.1</v>
       </c>
       <c r="U15">
-        <v>3.25</v>
+        <v>3</v>
       </c>
       <c r="V15">
         <v>0.4</v>
       </c>
       <c r="W15">
-        <v>63.4</v>
+        <v>54</v>
       </c>
       <c r="X15">
-        <v>4.21</v>
+        <v>3.58</v>
       </c>
       <c r="Y15">
-        <v>10.8</v>
+        <v>9.2</v>
       </c>
       <c r="Z15" t="str">
         <v>Ø12 a200</v>
       </c>
       <c r="AA15">
-        <v>0.66</v>
+        <v>0.84</v>
       </c>
       <c r="AB15">
-        <v>0.58</v>
+        <v>0.61</v>
       </c>
       <c r="AC15">
-        <v>0.93</v>
+        <v>0.99</v>
       </c>
       <c r="AD15">
-        <v>0.71</v>
+        <v>0.96</v>
       </c>
       <c r="AE15">
         <v>0.15</v>
@@ -19155,7 +19155,7 @@
         <v>0.62</v>
       </c>
       <c r="AG15">
-        <v>0.93</v>
+        <v>0.99</v>
       </c>
       <c r="AH15" t="str">
         <v>ĐẠT</v>
@@ -20254,7 +20254,7 @@
         <v>73.7</v>
       </c>
       <c r="G26">
-        <v>12.97</v>
+        <v>14.34</v>
       </c>
       <c r="H26" t="str">
         <v>B7-D23</v>
@@ -20266,13 +20266,13 @@
         <v>45.6</v>
       </c>
       <c r="K26">
-        <v>15.85</v>
+        <v>14.34</v>
       </c>
       <c r="L26">
-        <v>172.09</v>
+        <v>170.95</v>
       </c>
       <c r="M26">
-        <v>-80.6</v>
+        <v>-78.93</v>
       </c>
       <c r="N26">
         <v>378.3</v>
@@ -20290,10 +20290,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S26">
-        <v>25.2</v>
+        <v>25.1</v>
       </c>
       <c r="T26">
-        <v>54.3</v>
+        <v>53.2</v>
       </c>
       <c r="U26">
         <v>2.75</v>
@@ -20314,16 +20314,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA26">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
       <c r="AB26">
         <v>0.67</v>
       </c>
       <c r="AC26">
-        <v>0.89</v>
+        <v>0.87</v>
       </c>
       <c r="AD26">
-        <v>0.79</v>
+        <v>0.75</v>
       </c>
       <c r="AE26">
         <v>0.15</v>
@@ -20332,7 +20332,7 @@
         <v>0.62</v>
       </c>
       <c r="AG26">
-        <v>0.89</v>
+        <v>0.87</v>
       </c>
       <c r="AH26" t="str">
         <v>ĐẠT</v>
@@ -20361,7 +20361,7 @@
         <v>73.7</v>
       </c>
       <c r="G27">
-        <v>14.5</v>
+        <v>14.36</v>
       </c>
       <c r="H27" t="str">
         <v>B7-D32</v>
@@ -20373,13 +20373,13 @@
         <v>45.6</v>
       </c>
       <c r="K27">
-        <v>14.29</v>
+        <v>14.37</v>
       </c>
       <c r="L27">
-        <v>157.75</v>
+        <v>156.82</v>
       </c>
       <c r="M27">
-        <v>-78.99</v>
+        <v>-78.93</v>
       </c>
       <c r="N27">
         <v>378.3</v>
@@ -20397,10 +20397,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S27">
-        <v>26.2</v>
+        <v>25.1</v>
       </c>
       <c r="T27">
-        <v>53</v>
+        <v>53.1</v>
       </c>
       <c r="U27">
         <v>2.75</v>
@@ -20427,7 +20427,7 @@
         <v>0.67</v>
       </c>
       <c r="AC27">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="AD27">
         <v>0.75</v>
@@ -20439,7 +20439,7 @@
         <v>0.62</v>
       </c>
       <c r="AG27">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="AH27" t="str">
         <v>ĐẠT</v>
@@ -20468,7 +20468,7 @@
         <v>73.7</v>
       </c>
       <c r="G28">
-        <v>14.56</v>
+        <v>14.31</v>
       </c>
       <c r="H28" t="str">
         <v>B7-D19</v>
@@ -20480,13 +20480,13 @@
         <v>45.6</v>
       </c>
       <c r="K28">
-        <v>14.18</v>
+        <v>14.32</v>
       </c>
       <c r="L28">
-        <v>143.31</v>
+        <v>142.07</v>
       </c>
       <c r="M28">
-        <v>-78.94</v>
+        <v>-78.93</v>
       </c>
       <c r="N28">
         <v>378.3</v>
@@ -20504,10 +20504,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S28">
-        <v>26.9</v>
+        <v>25.1</v>
       </c>
       <c r="T28">
-        <v>53</v>
+        <v>53.3</v>
       </c>
       <c r="U28">
         <v>2.75</v>
@@ -20531,13 +20531,13 @@
         <v>0.73</v>
       </c>
       <c r="AB28">
-        <v>0.68</v>
+        <v>0.67</v>
       </c>
       <c r="AC28">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="AD28">
-        <v>0.77</v>
+        <v>0.75</v>
       </c>
       <c r="AE28">
         <v>0.15</v>
@@ -20546,7 +20546,7 @@
         <v>0.62</v>
       </c>
       <c r="AG28">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="AH28" t="str">
         <v>ĐẠT</v>
@@ -20575,7 +20575,7 @@
         <v>73.7</v>
       </c>
       <c r="G29">
-        <v>14.12</v>
+        <v>14.34</v>
       </c>
       <c r="H29" t="str">
         <v>B7-D31</v>
@@ -20587,13 +20587,13 @@
         <v>45.6</v>
       </c>
       <c r="K29">
-        <v>14.63</v>
+        <v>14.34</v>
       </c>
       <c r="L29">
-        <v>128.93</v>
+        <v>127.95</v>
       </c>
       <c r="M29">
-        <v>-79.36</v>
+        <v>-78.93</v>
       </c>
       <c r="N29">
         <v>378.3</v>
@@ -20611,10 +20611,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S29">
-        <v>25.9</v>
+        <v>25.1</v>
       </c>
       <c r="T29">
-        <v>53.3</v>
+        <v>53.2</v>
       </c>
       <c r="U29">
         <v>2.75</v>
@@ -20641,10 +20641,10 @@
         <v>0.67</v>
       </c>
       <c r="AC29">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="AD29">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="AE29">
         <v>0.15</v>
@@ -20653,7 +20653,7 @@
         <v>0.62</v>
       </c>
       <c r="AG29">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="AH29" t="str">
         <v>ĐẠT</v>
@@ -20682,7 +20682,7 @@
         <v>73.7</v>
       </c>
       <c r="G30">
-        <v>14.53</v>
+        <v>14.29</v>
       </c>
       <c r="H30" t="str">
         <v>B7-D22</v>
@@ -20694,13 +20694,13 @@
         <v>45.6</v>
       </c>
       <c r="K30">
-        <v>14.17</v>
+        <v>14.3</v>
       </c>
       <c r="L30">
-        <v>114.44</v>
+        <v>113.2</v>
       </c>
       <c r="M30">
-        <v>-78.94</v>
+        <v>-78.93</v>
       </c>
       <c r="N30">
         <v>378.3</v>
@@ -20718,10 +20718,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S30">
-        <v>26.9</v>
+        <v>25.1</v>
       </c>
       <c r="T30">
-        <v>53.1</v>
+        <v>53.3</v>
       </c>
       <c r="U30">
         <v>2.75</v>
@@ -20742,16 +20742,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA30">
-        <v>0.73</v>
+        <v>0.74</v>
       </c>
       <c r="AB30">
-        <v>0.68</v>
+        <v>0.67</v>
       </c>
       <c r="AC30">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="AD30">
-        <v>0.77</v>
+        <v>0.75</v>
       </c>
       <c r="AE30">
         <v>0.15</v>
@@ -20760,7 +20760,7 @@
         <v>0.62</v>
       </c>
       <c r="AG30">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="AH30" t="str">
         <v>ĐẠT</v>
@@ -20789,7 +20789,7 @@
         <v>87.3</v>
       </c>
       <c r="G31">
-        <v>22.11</v>
+        <v>21.31</v>
       </c>
       <c r="H31" t="str">
         <v>B6-D27</v>
@@ -20801,19 +20801,19 @@
         <v>40.8</v>
       </c>
       <c r="K31">
-        <v>20.76</v>
+        <v>21.3</v>
       </c>
       <c r="L31">
-        <v>371.71</v>
+        <v>369.3</v>
       </c>
       <c r="M31">
-        <v>-73.49</v>
+        <v>-73.82</v>
       </c>
       <c r="N31">
         <v>378.3</v>
       </c>
       <c r="O31">
-        <v>381.41</v>
+        <v>381.37</v>
       </c>
       <c r="P31">
         <v>1.7</v>
@@ -20825,40 +20825,40 @@
         <v>B5A-D13 căng, B6-D27 chùng (MN cao)</v>
       </c>
       <c r="S31">
-        <v>78.5</v>
+        <v>78.1</v>
       </c>
       <c r="T31">
-        <v>28.5</v>
+        <v>29.4</v>
       </c>
       <c r="U31">
-        <v>2.5</v>
+        <v>2.75</v>
       </c>
       <c r="V31">
         <v>0.4</v>
       </c>
       <c r="W31">
-        <v>37.5</v>
+        <v>45.4</v>
       </c>
       <c r="X31">
-        <v>2.48</v>
+        <v>3.01</v>
       </c>
       <c r="Y31">
-        <v>6.4</v>
+        <v>7.7</v>
       </c>
       <c r="Z31" t="str">
         <v>Ø12 a200</v>
       </c>
       <c r="AA31">
-        <v>0.61</v>
+        <v>0.56</v>
       </c>
       <c r="AB31">
-        <v>0.92</v>
+        <v>0.81</v>
       </c>
       <c r="AC31">
-        <v>0.94</v>
+        <v>0.84</v>
       </c>
       <c r="AD31">
-        <v>0.98</v>
+        <v>0.66</v>
       </c>
       <c r="AE31">
         <v>0.15</v>
@@ -20867,13 +20867,13 @@
         <v>0.62</v>
       </c>
       <c r="AG31">
-        <v>0.98</v>
+        <v>0.84</v>
       </c>
       <c r="AH31" t="str">
         <v>ĐẠT</v>
       </c>
       <c r="AI31" t="str">
-        <v>Đế dùng chung hai bè: hai tai neo; Địa hình IFC tại điểm này cao hơn đáy thiết kế 3,1 m: kiểm tra khảo sát / nạo vét trước khi đặt đế</v>
+        <v>Đế dùng chung hai bè: hai tai neo; Địa hình IFC tại điểm này cao hơn đáy thiết kế 3,1 m: kiểm tra khảo sát / nạo vét trước khi đặt đế; Đế lớn hơn đế mẫu</v>
       </c>
     </row>
     <row r="32">
@@ -21003,7 +21003,7 @@
         <v>87.3</v>
       </c>
       <c r="G33">
-        <v>25.58</v>
+        <v>21.46</v>
       </c>
       <c r="H33" t="str">
         <v>B6-D17</v>
@@ -21015,19 +21015,19 @@
         <v>40.8</v>
       </c>
       <c r="K33">
-        <v>22.08</v>
+        <v>21.45</v>
       </c>
       <c r="L33">
-        <v>337.83</v>
+        <v>346.24</v>
       </c>
       <c r="M33">
-        <v>-69.35</v>
+        <v>-75.68</v>
       </c>
       <c r="N33">
         <v>378.3</v>
       </c>
       <c r="O33">
-        <v>381.18</v>
+        <v>381.05</v>
       </c>
       <c r="P33">
         <v>1.7</v>
@@ -21036,13 +21036,13 @@
         <v>7.7</v>
       </c>
       <c r="R33" t="str">
-        <v>cả hai dây căng (MN cao)</v>
+        <v>B5A-D15 căng, B6-D17 chùng (MN cao)</v>
       </c>
       <c r="S33">
-        <v>67.4</v>
+        <v>78.1</v>
       </c>
       <c r="T33">
-        <v>36.1</v>
+        <v>29.2</v>
       </c>
       <c r="U33">
         <v>2.75</v>
@@ -21063,16 +21063,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA33">
-        <v>0.5</v>
+        <v>0.56</v>
       </c>
       <c r="AB33">
+        <v>0.81</v>
+      </c>
+      <c r="AC33">
         <v>0.83</v>
       </c>
-      <c r="AC33">
-        <v>0.87</v>
-      </c>
       <c r="AD33">
-        <v>0.74</v>
+        <v>0.65</v>
       </c>
       <c r="AE33">
         <v>0.15</v>
@@ -21081,13 +21081,13 @@
         <v>0.62</v>
       </c>
       <c r="AG33">
-        <v>0.87</v>
+        <v>0.83</v>
       </c>
       <c r="AH33" t="str">
         <v>ĐẠT</v>
       </c>
       <c r="AI33" t="str">
-        <v>Đế dùng chung hai bè: hai tai neo; Địa hình IFC tại điểm này cao hơn đáy thiết kế 2,9 m: kiểm tra khảo sát / nạo vét trước khi đặt đế; Đế lớn hơn đế mẫu</v>
+        <v>Đế dùng chung hai bè: hai tai neo; Địa hình IFC tại điểm này cao hơn đáy thiết kế 2,8 m: kiểm tra khảo sát / nạo vét trước khi đặt đế; Đế lớn hơn đế mẫu</v>
       </c>
     </row>
     <row r="34">
@@ -21110,7 +21110,7 @@
         <v>45.6</v>
       </c>
       <c r="G34">
-        <v>10.67</v>
+        <v>11.52</v>
       </c>
       <c r="H34" t="str">
         <v>B8-D31</v>
@@ -21122,13 +21122,13 @@
         <v>59.1</v>
       </c>
       <c r="K34">
-        <v>12.49</v>
+        <v>11.52</v>
       </c>
       <c r="L34">
-        <v>111.96</v>
+        <v>110.63</v>
       </c>
       <c r="M34">
-        <v>89.82</v>
+        <v>90.49</v>
       </c>
       <c r="N34">
         <v>378.3</v>
@@ -21146,10 +21146,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S34">
-        <v>16.2</v>
+        <v>11.5</v>
       </c>
       <c r="T34">
-        <v>54.7</v>
+        <v>55.2</v>
       </c>
       <c r="U34">
         <v>2.5</v>
@@ -21176,10 +21176,10 @@
         <v>0.59</v>
       </c>
       <c r="AC34">
-        <v>0.92</v>
+        <v>0.9</v>
       </c>
       <c r="AD34">
-        <v>0.95</v>
+        <v>0.89</v>
       </c>
       <c r="AE34">
         <v>0.15</v>
@@ -21188,7 +21188,7 @@
         <v>0.62</v>
       </c>
       <c r="AG34">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="AH34" t="str">
         <v>ĐẠT</v>
@@ -21217,7 +21217,7 @@
         <v>45.6</v>
       </c>
       <c r="G35">
-        <v>16.61</v>
+        <v>13.97</v>
       </c>
       <c r="H35" t="str">
         <v>B8-D32</v>
@@ -21229,13 +21229,13 @@
         <v>59.1</v>
       </c>
       <c r="K35">
-        <v>11.6</v>
+        <v>13.98</v>
       </c>
       <c r="L35">
         <v>130.63</v>
       </c>
       <c r="M35">
-        <v>93.62</v>
+        <v>90.49</v>
       </c>
       <c r="N35">
         <v>378.3</v>
@@ -21253,10 +21253,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S35">
-        <v>15</v>
+        <v>12.1</v>
       </c>
       <c r="T35">
-        <v>49</v>
+        <v>47.7</v>
       </c>
       <c r="U35">
         <v>2.5</v>
@@ -21277,16 +21277,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA35">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
       <c r="AB35">
         <v>0.59</v>
       </c>
       <c r="AC35">
-        <v>0.83</v>
+        <v>0.79</v>
       </c>
       <c r="AD35">
-        <v>0.74</v>
+        <v>0.65</v>
       </c>
       <c r="AE35">
         <v>0.15</v>
@@ -21295,7 +21295,7 @@
         <v>0.62</v>
       </c>
       <c r="AG35">
-        <v>0.83</v>
+        <v>0.79</v>
       </c>
       <c r="AH35" t="str">
         <v>ĐẠT</v>
@@ -21324,7 +21324,7 @@
         <v>45.6</v>
       </c>
       <c r="G36">
-        <v>8.79</v>
+        <v>11.75</v>
       </c>
       <c r="H36" t="str">
         <v>B8-D29</v>
@@ -21336,13 +21336,13 @@
         <v>59.1</v>
       </c>
       <c r="K36">
-        <v>14.78</v>
+        <v>11.75</v>
       </c>
       <c r="L36">
         <v>83.63</v>
       </c>
       <c r="M36">
-        <v>87.37</v>
+        <v>90.49</v>
       </c>
       <c r="N36">
         <v>378.3</v>
@@ -21360,10 +21360,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S36">
-        <v>19.1</v>
+        <v>11.6</v>
       </c>
       <c r="T36">
-        <v>54.5</v>
+        <v>54.4</v>
       </c>
       <c r="U36">
         <v>2.5</v>
@@ -21390,10 +21390,10 @@
         <v>0.59</v>
       </c>
       <c r="AC36">
-        <v>0.94</v>
+        <v>0.89</v>
       </c>
       <c r="AD36">
-        <v>0.98</v>
+        <v>0.87</v>
       </c>
       <c r="AE36">
         <v>0.15</v>
@@ -21402,7 +21402,7 @@
         <v>0.62</v>
       </c>
       <c r="AG36">
-        <v>0.98</v>
+        <v>0.89</v>
       </c>
       <c r="AH36" t="str">
         <v>ĐẠT</v>
@@ -21538,7 +21538,7 @@
         <v>59.1</v>
       </c>
       <c r="G38">
-        <v>12.14</v>
+        <v>11.49</v>
       </c>
       <c r="H38" t="str">
         <v>B9-D16</v>
@@ -21550,19 +21550,19 @@
         <v>30.9</v>
       </c>
       <c r="K38">
-        <v>14.24</v>
+        <v>11.49</v>
       </c>
       <c r="L38">
-        <v>115.24</v>
+        <v>121.79</v>
       </c>
       <c r="M38">
-        <v>293.32</v>
+        <v>292.95</v>
       </c>
       <c r="N38">
         <v>378.3</v>
       </c>
       <c r="O38">
-        <v>380.69</v>
+        <v>380.8</v>
       </c>
       <c r="P38">
         <v>1.7</v>
@@ -21574,10 +21574,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S38">
-        <v>43.6</v>
+        <v>24</v>
       </c>
       <c r="T38">
-        <v>43.9</v>
+        <v>47.6</v>
       </c>
       <c r="U38">
         <v>2.5</v>
@@ -21598,16 +21598,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA38">
-        <v>0.67</v>
+        <v>0.73</v>
       </c>
       <c r="AB38">
-        <v>0.87</v>
+        <v>0.59</v>
       </c>
       <c r="AC38">
-        <v>0.94</v>
+        <v>0.86</v>
       </c>
       <c r="AD38">
-        <v>0.98</v>
+        <v>0.82</v>
       </c>
       <c r="AE38">
         <v>0.15</v>
@@ -21616,13 +21616,13 @@
         <v>0.62</v>
       </c>
       <c r="AG38">
-        <v>0.98</v>
+        <v>0.86</v>
       </c>
       <c r="AH38" t="str">
         <v>ĐẠT</v>
       </c>
       <c r="AI38" t="str">
-        <v>Đế dùng chung hai bè: hai tai neo; Địa hình IFC tại điểm này cao hơn đáy thiết kế 2,4 m: kiểm tra khảo sát / nạo vét trước khi đặt đế</v>
+        <v>Đế dùng chung hai bè: hai tai neo; Địa hình IFC tại điểm này cao hơn đáy thiết kế 2,5 m: kiểm tra khảo sát / nạo vét trước khi đặt đế</v>
       </c>
     </row>
     <row r="39">
@@ -21684,7 +21684,7 @@
         <v>Bê tông đế</v>
       </c>
       <c r="B45">
-        <v>93.4</v>
+        <v>92.2</v>
       </c>
       <c r="C45" t="str">
         <v>m³</v>
@@ -21717,7 +21717,7 @@
         <v>Số đế cạnh B = 2,75 m</v>
       </c>
       <c r="B48">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C48" t="str">
         <v>đế</v>
@@ -21739,7 +21739,7 @@
         <v>Số đế cạnh B = 3,25 m</v>
       </c>
       <c r="B50">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C50" t="str">
         <v>đế</v>
@@ -21750,7 +21750,7 @@
         <v>Số đế mà địa hình IFC cao hơn đáy thiết kế trên 0,5 m (cần kiểm tra khảo sát / nạo vét)</v>
       </c>
       <c r="B51">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C51" t="str">
         <v>đế</v>
@@ -25490,19 +25490,19 @@
         <v>Chuyển từ neo đáy</v>
       </c>
       <c r="F50">
-        <v>-41.3</v>
+        <v>-35.8</v>
       </c>
       <c r="G50">
-        <v>-149.57</v>
+        <v>-179.26</v>
       </c>
       <c r="H50">
-        <v>384.08</v>
+        <v>385.08</v>
       </c>
       <c r="I50">
-        <v>37.5</v>
+        <v>58</v>
       </c>
       <c r="J50">
-        <v>232</v>
+        <v>204.5</v>
       </c>
       <c r="K50">
         <v>1</v>
@@ -25538,13 +25538,13 @@
         <v>H-8 Cao độ chốt cáp so với yêu cầu thiết kế cọc</v>
       </c>
       <c r="V50">
-        <v>-5.8</v>
+        <v>-4.8</v>
       </c>
       <c r="W50">
-        <v>3.3</v>
+        <v>1.2</v>
       </c>
       <c r="X50" t="str">
-        <v>CÓ</v>
+        <v>không</v>
       </c>
       <c r="Y50" t="str">
         <v>CÓ</v>
@@ -25553,7 +25553,7 @@
         <v>ĐẠT</v>
       </c>
       <c r="AA50" t="str">
-        <v>Chuyển từ neo đáy sang cọc khoan nhồi (vị trí ven bờ); Mặt đất tại cọc thấp hơn MNDB: thi công mùa nước thấp, có ống vách; Đầu cọc ngập khi hồ ở MNLKT: bản mã, tai neo cần chống gỉ</v>
+        <v>Chuyển từ neo đáy sang cọc khoan nhồi (vị trí ven bờ); Đầu cọc ngập khi hồ ở MNLKT: bản mã, tai neo cần chống gỉ</v>
       </c>
     </row>
     <row r="51">
@@ -31217,19 +31217,19 @@
         <v>Chuyển từ neo đáy</v>
       </c>
       <c r="F119">
-        <v>419.48</v>
+        <v>423.01</v>
       </c>
       <c r="G119">
-        <v>-154.12</v>
+        <v>-168.16</v>
       </c>
       <c r="H119">
-        <v>384.2</v>
+        <v>388.57</v>
       </c>
       <c r="I119">
-        <v>49.52</v>
+        <v>58.5</v>
       </c>
       <c r="J119">
-        <v>107.9</v>
+        <v>120</v>
       </c>
       <c r="K119">
         <v>1</v>
@@ -31265,22 +31265,22 @@
         <v>H-8 Cao độ chốt cáp so với yêu cầu thiết kế cọc</v>
       </c>
       <c r="V119">
-        <v>-4.6</v>
+        <v>-8.1</v>
       </c>
       <c r="W119">
-        <v>2.4</v>
+        <v>-2.3</v>
       </c>
       <c r="X119" t="str">
-        <v>CÓ</v>
+        <v>không</v>
       </c>
       <c r="Y119" t="str">
-        <v>CÓ</v>
+        <v>không</v>
       </c>
       <c r="Z119" t="str">
         <v>ĐẠT</v>
       </c>
       <c r="AA119" t="str">
-        <v>Chuyển từ neo đáy sang cọc khoan nhồi (vị trí ven bờ); Mặt đất tại cọc thấp hơn MNDB: thi công mùa nước thấp, có ống vách; Đầu cọc ngập khi hồ ở MNLKT: bản mã, tai neo cần chống gỉ</v>
+        <v>Chuyển từ neo đáy sang cọc khoan nhồi (vị trí ven bờ)</v>
       </c>
     </row>
     <row r="120">
@@ -31300,19 +31300,19 @@
         <v>Chuyển từ neo đáy</v>
       </c>
       <c r="F120">
-        <v>420.28</v>
+        <v>418.19</v>
       </c>
       <c r="G120">
-        <v>-149.28</v>
+        <v>-162.96</v>
       </c>
       <c r="H120">
-        <v>384.75</v>
+        <v>384</v>
       </c>
       <c r="I120">
-        <v>35</v>
+        <v>39.5</v>
       </c>
       <c r="J120">
-        <v>107.2</v>
+        <v>127.5</v>
       </c>
       <c r="K120">
         <v>1</v>
@@ -31348,13 +31348,13 @@
         <v>H-8 Cao độ chốt cáp so với yêu cầu thiết kế cọc</v>
       </c>
       <c r="V120">
-        <v>-7.3</v>
+        <v>-5.4</v>
       </c>
       <c r="W120">
-        <v>2.5</v>
+        <v>3.3</v>
       </c>
       <c r="X120" t="str">
-        <v>không</v>
+        <v>CÓ</v>
       </c>
       <c r="Y120" t="str">
         <v>CÓ</v>
@@ -31363,7 +31363,7 @@
         <v>ĐẠT</v>
       </c>
       <c r="AA120" t="str">
-        <v>Chuyển từ neo đáy sang cọc khoan nhồi (vị trí ven bờ); Đầu cọc ngập khi hồ ở MNLKT: bản mã, tai neo cần chống gỉ</v>
+        <v>Chuyển từ neo đáy sang cọc khoan nhồi (vị trí ven bờ); Mặt đất tại cọc thấp hơn MNDB: thi công mùa nước thấp, có ống vách; Đầu cọc ngập khi hồ ở MNLKT: bản mã, tai neo cần chống gỉ</v>
       </c>
     </row>
     <row r="121">
@@ -35616,19 +35616,19 @@
         <v>Chuyển từ neo đáy</v>
       </c>
       <c r="F172">
-        <v>76.46</v>
+        <v>81.73</v>
       </c>
       <c r="G172">
-        <v>-76.01</v>
+        <v>-97.29</v>
       </c>
       <c r="H172">
-        <v>384.07</v>
+        <v>384.1</v>
       </c>
       <c r="I172">
-        <v>26.5</v>
+        <v>37.5</v>
       </c>
       <c r="J172">
-        <v>245</v>
+        <v>210</v>
       </c>
       <c r="K172">
         <v>1</v>
@@ -35664,10 +35664,10 @@
         <v>H-8 Cao độ chốt cáp so với yêu cầu thiết kế cọc</v>
       </c>
       <c r="V172">
-        <v>-8.2</v>
+        <v>-5.9</v>
       </c>
       <c r="W172">
-        <v>4.7</v>
+        <v>3.3</v>
       </c>
       <c r="X172" t="str">
         <v>CÓ</v>
@@ -37940,19 +37940,19 @@
         <v>Chuyển từ neo đáy</v>
       </c>
       <c r="F200">
-        <v>41.03</v>
+        <v>47.33</v>
       </c>
       <c r="G200">
-        <v>92.56</v>
+        <v>71.85</v>
       </c>
       <c r="H200">
-        <v>384.03</v>
+        <v>384.01</v>
       </c>
       <c r="I200">
-        <v>27</v>
+        <v>35.5</v>
       </c>
       <c r="J200">
-        <v>250</v>
+        <v>212.5</v>
       </c>
       <c r="K200">
         <v>1</v>
@@ -37988,10 +37988,10 @@
         <v>H-8 Cao độ chốt cáp so với yêu cầu thiết kế cọc</v>
       </c>
       <c r="V200">
-        <v>-8</v>
+        <v>-6</v>
       </c>
       <c r="W200">
-        <v>4.7</v>
+        <v>3.6</v>
       </c>
       <c r="X200" t="str">
         <v>CÓ</v>
@@ -41136,7 +41136,7 @@
         <v>Dây neo bờ dài nhất</v>
       </c>
       <c r="B244">
-        <v>58.4</v>
+        <v>58.5</v>
       </c>
       <c r="C244" t="str">
         <v>m</v>
@@ -41147,7 +41147,7 @@
         <v>Số điểm có mặt đất tại cọc thấp hơn MNDB</v>
       </c>
       <c r="B245">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C245" t="str">
         <v>điểm</v>
@@ -41158,7 +41158,7 @@
         <v>Số điểm có đầu cọc ngập khi hồ ở MNLKT</v>
       </c>
       <c r="B246">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C246" t="str">
         <v>điểm</v>

</xml_diff>

<commit_message>
feat: bang tinh va thuyet minh phuong an chot (coc khoan nhoi ven bo + de BTCT vit xoan)
- finalDesignWorkbook: mot nguon cho bang tinh Excel 9 sheet, thuyet minh tren web va sheet bao gia
- nut "Bang Tinh" o Header, tab Bao cao va Muc 10; muc thuyet minh ca 9 be o dau tab Bao cao
- tinh de: bich be cao hon mat nuoc 0,35 m (cleatHeight_m) -> HV-DV009 tu 3,0 len 3,25 m, 92,8 m3
- xuat lai ban ve DXF/DWG, bang thong ke va file dinh kem tren web; them file bang tinh dinh kem

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/mat-bang-neo-9-be/bang_thong_ke_neo_9_be.xlsx
+++ b/docs/mat-bang-neo-9-be/bang_thong_ke_neo_9_be.xlsx
@@ -15014,13 +15014,13 @@
         <v>30.2</v>
       </c>
       <c r="R6">
-        <v>0.44</v>
+        <v>0.45</v>
       </c>
       <c r="S6">
         <v>0.27</v>
       </c>
       <c r="T6">
-        <v>0.44</v>
+        <v>0.46</v>
       </c>
       <c r="U6">
         <v>0</v>
@@ -15088,13 +15088,13 @@
         <v>30.2</v>
       </c>
       <c r="R7">
-        <v>0.47</v>
+        <v>0.49</v>
       </c>
       <c r="S7">
         <v>0.27</v>
       </c>
       <c r="T7">
-        <v>0.47</v>
+        <v>0.49</v>
       </c>
       <c r="U7">
         <v>0</v>
@@ -15162,16 +15162,16 @@
         <v>38.6</v>
       </c>
       <c r="R8">
-        <v>0.59</v>
+        <v>0.61</v>
       </c>
       <c r="S8">
         <v>0.36</v>
       </c>
       <c r="T8">
-        <v>0.63</v>
+        <v>0.65</v>
       </c>
       <c r="U8">
-        <v>0.29</v>
+        <v>0.33</v>
       </c>
       <c r="V8">
         <v>0.15</v>
@@ -15236,16 +15236,16 @@
         <v>38.6</v>
       </c>
       <c r="R9">
-        <v>0.63</v>
+        <v>0.65</v>
       </c>
       <c r="S9">
         <v>0.36</v>
       </c>
       <c r="T9">
-        <v>0.67</v>
+        <v>0.69</v>
       </c>
       <c r="U9">
-        <v>0.38</v>
+        <v>0.42</v>
       </c>
       <c r="V9">
         <v>0.15</v>
@@ -15310,16 +15310,16 @@
         <v>38.6</v>
       </c>
       <c r="R10">
-        <v>0.46</v>
+        <v>0.47</v>
       </c>
       <c r="S10">
-        <v>0.37</v>
+        <v>0.36</v>
       </c>
       <c r="T10">
-        <v>0.51</v>
+        <v>0.52</v>
       </c>
       <c r="U10">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="V10">
         <v>0.15</v>
@@ -15384,16 +15384,16 @@
         <v>73.7</v>
       </c>
       <c r="R11">
-        <v>0.77</v>
+        <v>0.79</v>
       </c>
       <c r="S11">
         <v>0.55</v>
       </c>
       <c r="T11">
-        <v>0.92</v>
+        <v>0.94</v>
       </c>
       <c r="U11">
-        <v>0.68</v>
+        <v>0.74</v>
       </c>
       <c r="V11">
         <v>0.15</v>
@@ -15458,16 +15458,16 @@
         <v>73.7</v>
       </c>
       <c r="R12">
-        <v>0.73</v>
+        <v>0.75</v>
       </c>
       <c r="S12">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="T12">
-        <v>0.91</v>
+        <v>0.94</v>
       </c>
       <c r="U12">
-        <v>0.93</v>
+        <v>0.99</v>
       </c>
       <c r="V12">
         <v>0.15</v>
@@ -15532,16 +15532,16 @@
         <v>73.7</v>
       </c>
       <c r="R13">
-        <v>0.78</v>
+        <v>0.8</v>
       </c>
       <c r="S13">
         <v>0.67</v>
       </c>
       <c r="T13">
-        <v>0.94</v>
+        <v>0.97</v>
       </c>
       <c r="U13">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="V13">
         <v>0.15</v>
@@ -15582,19 +15582,19 @@
         <v>135.9</v>
       </c>
       <c r="J14">
-        <v>3</v>
+        <v>3.25</v>
       </c>
       <c r="K14">
         <v>0.4</v>
       </c>
       <c r="L14">
-        <v>3.58</v>
+        <v>4.21</v>
       </c>
       <c r="M14">
-        <v>165</v>
+        <v>202</v>
       </c>
       <c r="N14">
-        <v>9.2</v>
+        <v>10.8</v>
       </c>
       <c r="O14">
         <v>4</v>
@@ -15606,16 +15606,16 @@
         <v>73.7</v>
       </c>
       <c r="R14">
-        <v>0.84</v>
+        <v>0.78</v>
       </c>
       <c r="S14">
-        <v>0.61</v>
+        <v>0.55</v>
       </c>
       <c r="T14">
-        <v>0.99</v>
+        <v>0.93</v>
       </c>
       <c r="U14">
-        <v>0.96</v>
+        <v>0.71</v>
       </c>
       <c r="V14">
         <v>0.15</v>
@@ -15680,16 +15680,16 @@
         <v>87.3</v>
       </c>
       <c r="R15">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="S15">
         <v>0.81</v>
       </c>
       <c r="T15">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="U15">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="V15">
         <v>0.15</v>
@@ -15754,16 +15754,16 @@
         <v>87.3</v>
       </c>
       <c r="R16">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="S16">
         <v>0.81</v>
       </c>
       <c r="T16">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="U16">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="V16">
         <v>0.15</v>
@@ -15828,16 +15828,16 @@
         <v>87.3</v>
       </c>
       <c r="R17">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="S17">
         <v>0.81</v>
       </c>
       <c r="T17">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="U17">
-        <v>0.68</v>
+        <v>0.72</v>
       </c>
       <c r="V17">
         <v>0.15</v>
@@ -15902,16 +15902,16 @@
         <v>87.3</v>
       </c>
       <c r="R18">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="S18">
         <v>0.81</v>
       </c>
       <c r="T18">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="U18">
-        <v>0.68</v>
+        <v>0.72</v>
       </c>
       <c r="V18">
         <v>0.15</v>
@@ -15976,16 +15976,16 @@
         <v>87.3</v>
       </c>
       <c r="R19">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="S19">
         <v>0.81</v>
       </c>
       <c r="T19">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="U19">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="V19">
         <v>0.15</v>
@@ -16050,16 +16050,16 @@
         <v>87.3</v>
       </c>
       <c r="R20">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="S20">
         <v>0.81</v>
       </c>
       <c r="T20">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="U20">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="V20">
         <v>0.15</v>
@@ -16124,16 +16124,16 @@
         <v>87.3</v>
       </c>
       <c r="R21">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="S21">
         <v>0.81</v>
       </c>
       <c r="T21">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="U21">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="V21">
         <v>0.15</v>
@@ -16198,16 +16198,16 @@
         <v>87.3</v>
       </c>
       <c r="R22">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="S22">
         <v>0.81</v>
       </c>
       <c r="T22">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="U22">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="V22">
         <v>0.15</v>
@@ -16272,16 +16272,16 @@
         <v>87.3</v>
       </c>
       <c r="R23">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="S23">
         <v>0.81</v>
       </c>
       <c r="T23">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="U23">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="V23">
         <v>0.15</v>
@@ -16346,16 +16346,16 @@
         <v>87.3</v>
       </c>
       <c r="R24">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="S24">
         <v>0.81</v>
       </c>
       <c r="T24">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="U24">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="V24">
         <v>0.15</v>
@@ -16420,16 +16420,16 @@
         <v>73.7</v>
       </c>
       <c r="R25">
-        <v>0.73</v>
+        <v>0.76</v>
       </c>
       <c r="S25">
         <v>0.67</v>
       </c>
       <c r="T25">
-        <v>0.87</v>
+        <v>0.9</v>
       </c>
       <c r="U25">
-        <v>0.75</v>
+        <v>0.81</v>
       </c>
       <c r="V25">
         <v>0.15</v>
@@ -16494,16 +16494,16 @@
         <v>73.7</v>
       </c>
       <c r="R26">
-        <v>0.73</v>
+        <v>0.76</v>
       </c>
       <c r="S26">
         <v>0.67</v>
       </c>
       <c r="T26">
-        <v>0.87</v>
+        <v>0.9</v>
       </c>
       <c r="U26">
-        <v>0.75</v>
+        <v>0.81</v>
       </c>
       <c r="V26">
         <v>0.15</v>
@@ -16568,16 +16568,16 @@
         <v>73.7</v>
       </c>
       <c r="R27">
-        <v>0.73</v>
+        <v>0.76</v>
       </c>
       <c r="S27">
         <v>0.67</v>
       </c>
       <c r="T27">
-        <v>0.87</v>
+        <v>0.9</v>
       </c>
       <c r="U27">
-        <v>0.75</v>
+        <v>0.82</v>
       </c>
       <c r="V27">
         <v>0.15</v>
@@ -16642,16 +16642,16 @@
         <v>73.7</v>
       </c>
       <c r="R28">
-        <v>0.73</v>
+        <v>0.76</v>
       </c>
       <c r="S28">
         <v>0.67</v>
       </c>
       <c r="T28">
-        <v>0.87</v>
+        <v>0.9</v>
       </c>
       <c r="U28">
-        <v>0.75</v>
+        <v>0.81</v>
       </c>
       <c r="V28">
         <v>0.15</v>
@@ -16716,16 +16716,16 @@
         <v>73.7</v>
       </c>
       <c r="R29">
-        <v>0.74</v>
+        <v>0.76</v>
       </c>
       <c r="S29">
         <v>0.67</v>
       </c>
       <c r="T29">
-        <v>0.87</v>
+        <v>0.9</v>
       </c>
       <c r="U29">
-        <v>0.75</v>
+        <v>0.82</v>
       </c>
       <c r="V29">
         <v>0.15</v>
@@ -16790,16 +16790,16 @@
         <v>87.3</v>
       </c>
       <c r="R30">
-        <v>0.56</v>
+        <v>0.59</v>
       </c>
       <c r="S30">
         <v>0.81</v>
       </c>
       <c r="T30">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="U30">
-        <v>0.66</v>
+        <v>0.7</v>
       </c>
       <c r="V30">
         <v>0.15</v>
@@ -16864,16 +16864,16 @@
         <v>87.3</v>
       </c>
       <c r="R31">
-        <v>0.61</v>
+        <v>0.64</v>
       </c>
       <c r="S31">
-        <v>0.81</v>
+        <v>0.85</v>
       </c>
       <c r="T31">
-        <v>0.87</v>
+        <v>0.89</v>
       </c>
       <c r="U31">
-        <v>0.74</v>
+        <v>0.78</v>
       </c>
       <c r="V31">
         <v>0.15</v>
@@ -16938,16 +16938,16 @@
         <v>87.3</v>
       </c>
       <c r="R32">
-        <v>0.56</v>
+        <v>0.58</v>
       </c>
       <c r="S32">
         <v>0.81</v>
       </c>
       <c r="T32">
-        <v>0.83</v>
+        <v>0.85</v>
       </c>
       <c r="U32">
-        <v>0.65</v>
+        <v>0.69</v>
       </c>
       <c r="V32">
         <v>0.15</v>
@@ -17012,16 +17012,16 @@
         <v>59.1</v>
       </c>
       <c r="R33">
-        <v>0.84</v>
+        <v>0.87</v>
       </c>
       <c r="S33">
         <v>0.59</v>
       </c>
       <c r="T33">
-        <v>0.9</v>
+        <v>0.92</v>
       </c>
       <c r="U33">
-        <v>0.89</v>
+        <v>0.95</v>
       </c>
       <c r="V33">
         <v>0.15</v>
@@ -17086,16 +17086,16 @@
         <v>59.1</v>
       </c>
       <c r="R34">
-        <v>0.73</v>
+        <v>0.76</v>
       </c>
       <c r="S34">
         <v>0.59</v>
       </c>
       <c r="T34">
-        <v>0.79</v>
+        <v>0.81</v>
       </c>
       <c r="U34">
-        <v>0.65</v>
+        <v>0.71</v>
       </c>
       <c r="V34">
         <v>0.15</v>
@@ -17160,16 +17160,16 @@
         <v>59.1</v>
       </c>
       <c r="R35">
-        <v>0.83</v>
+        <v>0.86</v>
       </c>
       <c r="S35">
         <v>0.59</v>
       </c>
       <c r="T35">
-        <v>0.89</v>
+        <v>0.91</v>
       </c>
       <c r="U35">
-        <v>0.87</v>
+        <v>0.93</v>
       </c>
       <c r="V35">
         <v>0.15</v>
@@ -17234,16 +17234,16 @@
         <v>59.1</v>
       </c>
       <c r="R36">
-        <v>0.86</v>
+        <v>0.89</v>
       </c>
       <c r="S36">
-        <v>0.59</v>
+        <v>0.58</v>
       </c>
       <c r="T36">
-        <v>0.91</v>
+        <v>0.94</v>
       </c>
       <c r="U36">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="V36">
         <v>0.15</v>
@@ -17308,16 +17308,16 @@
         <v>59.1</v>
       </c>
       <c r="R37">
-        <v>0.73</v>
+        <v>0.75</v>
       </c>
       <c r="S37">
         <v>0.59</v>
       </c>
       <c r="T37">
-        <v>0.86</v>
+        <v>0.89</v>
       </c>
       <c r="U37">
-        <v>0.82</v>
+        <v>0.87</v>
       </c>
       <c r="V37">
         <v>0.15</v>
@@ -17377,7 +17377,7 @@
         <v>Tổng bê tông đế</v>
       </c>
       <c r="B43">
-        <v>92.2</v>
+        <v>92.8</v>
       </c>
       <c r="C43" t="str">
         <v>m³</v>
@@ -17388,7 +17388,7 @@
         <v>Tổng thép bản đế (ước tính)</v>
       </c>
       <c r="B44">
-        <v>4.36</v>
+        <v>4.4</v>
       </c>
       <c r="C44" t="str">
         <v>tấn</v>
@@ -17562,25 +17562,25 @@
         <v>Ø12 a200</v>
       </c>
       <c r="F4">
-        <v>4.8</v>
+        <v>6.6</v>
       </c>
       <c r="G4">
-        <v>29.7</v>
+        <v>31</v>
       </c>
       <c r="H4">
-        <v>30.1</v>
+        <v>30</v>
       </c>
       <c r="I4">
-        <v>15</v>
+        <v>15.6</v>
       </c>
       <c r="J4">
-        <v>0.23</v>
+        <v>0.24</v>
       </c>
       <c r="K4">
         <v>0.33</v>
       </c>
       <c r="L4">
-        <v>0.39</v>
+        <v>0.4</v>
       </c>
       <c r="M4">
         <v>0</v>
@@ -17615,25 +17615,25 @@
         <v>Ø12 a200</v>
       </c>
       <c r="F5">
-        <v>6</v>
+        <v>8.2</v>
       </c>
       <c r="G5">
-        <v>36.5</v>
+        <v>37.9</v>
       </c>
       <c r="H5">
-        <v>27.6</v>
+        <v>27.5</v>
       </c>
       <c r="I5">
-        <v>16.5</v>
+        <v>17</v>
       </c>
       <c r="J5">
-        <v>0.25</v>
+        <v>0.26</v>
       </c>
       <c r="K5">
         <v>0.3</v>
       </c>
       <c r="L5">
-        <v>0.39</v>
+        <v>0.4</v>
       </c>
       <c r="M5">
         <v>0</v>
@@ -17668,28 +17668,28 @@
         <v>Ø12 a200</v>
       </c>
       <c r="F6">
-        <v>6</v>
+        <v>8.2</v>
       </c>
       <c r="G6">
-        <v>36.5</v>
+        <v>37.9</v>
       </c>
       <c r="H6">
-        <v>38.4</v>
+        <v>38.2</v>
       </c>
       <c r="I6">
-        <v>23</v>
+        <v>23.7</v>
       </c>
       <c r="J6">
-        <v>0.35</v>
+        <v>0.36</v>
       </c>
       <c r="K6">
         <v>0.42</v>
       </c>
       <c r="L6">
-        <v>0.54</v>
+        <v>0.55</v>
       </c>
       <c r="M6">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="N6">
         <v>0.15</v>
@@ -17721,28 +17721,28 @@
         <v>Ø12 a200</v>
       </c>
       <c r="F7">
-        <v>5.8</v>
+        <v>8</v>
       </c>
       <c r="G7">
-        <v>35.6</v>
+        <v>37</v>
       </c>
       <c r="H7">
-        <v>73.3</v>
+        <v>73</v>
       </c>
       <c r="I7">
-        <v>42.8</v>
+        <v>44.3</v>
       </c>
       <c r="J7">
-        <v>0.59</v>
+        <v>0.61</v>
       </c>
       <c r="K7">
         <v>0.72</v>
       </c>
       <c r="L7">
-        <v>0.92</v>
+        <v>0.94</v>
       </c>
       <c r="M7">
-        <v>0.87</v>
+        <v>0.9</v>
       </c>
       <c r="N7">
         <v>0.15</v>
@@ -17774,28 +17774,28 @@
         <v>Ø12 a200</v>
       </c>
       <c r="F8">
-        <v>2.8</v>
+        <v>3.9</v>
       </c>
       <c r="G8">
-        <v>19.1</v>
+        <v>20</v>
       </c>
       <c r="H8">
-        <v>87.2</v>
+        <v>87.1</v>
       </c>
       <c r="I8">
-        <v>28.6</v>
+        <v>29.9</v>
       </c>
       <c r="J8">
-        <v>0.39</v>
+        <v>0.41</v>
       </c>
       <c r="K8">
         <v>0.86</v>
       </c>
       <c r="L8">
-        <v>0.85</v>
+        <v>0.87</v>
       </c>
       <c r="M8">
-        <v>0.69</v>
+        <v>0.73</v>
       </c>
       <c r="N8">
         <v>0.15</v>
@@ -17827,28 +17827,28 @@
         <v>Ø12 a200</v>
       </c>
       <c r="F9">
-        <v>4.8</v>
+        <v>6.6</v>
       </c>
       <c r="G9">
-        <v>30.5</v>
+        <v>31.8</v>
       </c>
       <c r="H9">
-        <v>45.4</v>
+        <v>45.3</v>
       </c>
       <c r="I9">
-        <v>23.1</v>
+        <v>24</v>
       </c>
       <c r="J9">
-        <v>0.35</v>
+        <v>0.37</v>
       </c>
       <c r="K9">
-        <v>0.5</v>
+        <v>0.49</v>
       </c>
       <c r="L9">
-        <v>0.6</v>
+        <v>0.61</v>
       </c>
       <c r="M9">
-        <v>0.22</v>
+        <v>0.25</v>
       </c>
       <c r="N9">
         <v>0.15</v>
@@ -17880,25 +17880,25 @@
         <v>Ø12 a200</v>
       </c>
       <c r="F10">
-        <v>2.8</v>
+        <v>3.9</v>
       </c>
       <c r="G10">
-        <v>19.1</v>
+        <v>20</v>
       </c>
       <c r="H10">
-        <v>40.8</v>
+        <v>40.7</v>
       </c>
       <c r="I10">
-        <v>13.4</v>
+        <v>14</v>
       </c>
       <c r="J10">
-        <v>0.2</v>
+        <v>0.21</v>
       </c>
       <c r="K10">
         <v>0.44</v>
       </c>
       <c r="L10">
-        <v>0.45</v>
+        <v>0.46</v>
       </c>
       <c r="M10">
         <v>0</v>
@@ -17933,28 +17933,28 @@
         <v>Ø12 a200</v>
       </c>
       <c r="F11">
-        <v>4.8</v>
+        <v>6.6</v>
       </c>
       <c r="G11">
-        <v>30.5</v>
+        <v>31.8</v>
       </c>
       <c r="H11">
-        <v>58.9</v>
+        <v>58.7</v>
       </c>
       <c r="I11">
-        <v>30</v>
+        <v>31.1</v>
       </c>
       <c r="J11">
-        <v>0.46</v>
+        <v>0.48</v>
       </c>
       <c r="K11">
         <v>0.64</v>
       </c>
       <c r="L11">
-        <v>0.78</v>
+        <v>0.79</v>
       </c>
       <c r="M11">
-        <v>0.63</v>
+        <v>0.66</v>
       </c>
       <c r="N11">
         <v>0.15</v>
@@ -17986,22 +17986,22 @@
         <v>Ø12 a200</v>
       </c>
       <c r="F12">
-        <v>4.8</v>
+        <v>6.5</v>
       </c>
       <c r="G12">
-        <v>30.3</v>
+        <v>31.6</v>
       </c>
       <c r="H12">
-        <v>30.8</v>
+        <v>30.7</v>
       </c>
       <c r="I12">
-        <v>15.6</v>
+        <v>16.2</v>
       </c>
       <c r="J12">
-        <v>0.24</v>
+        <v>0.25</v>
       </c>
       <c r="K12">
-        <v>0.34</v>
+        <v>0.33</v>
       </c>
       <c r="L12">
         <v>0.41</v>
@@ -18031,7 +18031,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI51"/>
+  <dimension ref="A1:AI50"/>
   <cols>
     <col min="1" max="1" width="5.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -18258,10 +18258,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S7">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
       <c r="T7">
-        <v>28.7</v>
+        <v>29.7</v>
       </c>
       <c r="U7">
         <v>2.5</v>
@@ -18282,13 +18282,13 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA7">
-        <v>0.44</v>
+        <v>0.45</v>
       </c>
       <c r="AB7">
         <v>0.27</v>
       </c>
       <c r="AC7">
-        <v>0.44</v>
+        <v>0.46</v>
       </c>
       <c r="AD7">
         <v>0</v>
@@ -18368,7 +18368,7 @@
         <v>2.1</v>
       </c>
       <c r="T8">
-        <v>31</v>
+        <v>32.1</v>
       </c>
       <c r="U8">
         <v>2.5</v>
@@ -18389,13 +18389,13 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA8">
-        <v>0.47</v>
+        <v>0.49</v>
       </c>
       <c r="AB8">
         <v>0.27</v>
       </c>
       <c r="AC8">
-        <v>0.47</v>
+        <v>0.49</v>
       </c>
       <c r="AD8">
         <v>0</v>
@@ -18472,10 +18472,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S9">
-        <v>8.9</v>
+        <v>8.7</v>
       </c>
       <c r="T9">
-        <v>38.4</v>
+        <v>39.7</v>
       </c>
       <c r="U9">
         <v>2.5</v>
@@ -18496,16 +18496,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA9">
-        <v>0.59</v>
+        <v>0.61</v>
       </c>
       <c r="AB9">
         <v>0.36</v>
       </c>
       <c r="AC9">
-        <v>0.63</v>
+        <v>0.65</v>
       </c>
       <c r="AD9">
-        <v>0.29</v>
+        <v>0.33</v>
       </c>
       <c r="AE9">
         <v>0.15</v>
@@ -18514,7 +18514,7 @@
         <v>0.62</v>
       </c>
       <c r="AG9">
-        <v>0.63</v>
+        <v>0.65</v>
       </c>
       <c r="AH9" t="str">
         <v>ĐẠT</v>
@@ -18579,10 +18579,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S10">
-        <v>8.5</v>
+        <v>8.4</v>
       </c>
       <c r="T10">
-        <v>41.3</v>
+        <v>42.5</v>
       </c>
       <c r="U10">
         <v>2.5</v>
@@ -18603,16 +18603,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA10">
-        <v>0.63</v>
+        <v>0.65</v>
       </c>
       <c r="AB10">
         <v>0.36</v>
       </c>
       <c r="AC10">
-        <v>0.67</v>
+        <v>0.69</v>
       </c>
       <c r="AD10">
-        <v>0.38</v>
+        <v>0.42</v>
       </c>
       <c r="AE10">
         <v>0.15</v>
@@ -18621,7 +18621,7 @@
         <v>0.62</v>
       </c>
       <c r="AG10">
-        <v>0.67</v>
+        <v>0.69</v>
       </c>
       <c r="AH10" t="str">
         <v>ĐẠT</v>
@@ -18686,10 +18686,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S11">
-        <v>9.7</v>
+        <v>9.6</v>
       </c>
       <c r="T11">
-        <v>29.8</v>
+        <v>31</v>
       </c>
       <c r="U11">
         <v>2.5</v>
@@ -18710,16 +18710,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA11">
-        <v>0.46</v>
+        <v>0.47</v>
       </c>
       <c r="AB11">
-        <v>0.37</v>
+        <v>0.36</v>
       </c>
       <c r="AC11">
-        <v>0.51</v>
+        <v>0.52</v>
       </c>
       <c r="AD11">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="AE11">
         <v>0.15</v>
@@ -18793,10 +18793,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S12">
-        <v>27.8</v>
+        <v>27.3</v>
       </c>
       <c r="T12">
-        <v>68.2</v>
+        <v>70.3</v>
       </c>
       <c r="U12">
         <v>3.25</v>
@@ -18817,16 +18817,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA12">
-        <v>0.77</v>
+        <v>0.79</v>
       </c>
       <c r="AB12">
         <v>0.55</v>
       </c>
       <c r="AC12">
-        <v>0.92</v>
+        <v>0.94</v>
       </c>
       <c r="AD12">
-        <v>0.68</v>
+        <v>0.74</v>
       </c>
       <c r="AE12">
         <v>0.15</v>
@@ -18835,7 +18835,7 @@
         <v>0.62</v>
       </c>
       <c r="AG12">
-        <v>0.92</v>
+        <v>0.94</v>
       </c>
       <c r="AH12" t="str">
         <v>ĐẠT</v>
@@ -18900,10 +18900,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S13">
-        <v>31.7</v>
+        <v>31.5</v>
       </c>
       <c r="T13">
-        <v>47.5</v>
+        <v>49.4</v>
       </c>
       <c r="U13">
         <v>2.5</v>
@@ -18924,16 +18924,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA13">
-        <v>0.73</v>
+        <v>0.75</v>
       </c>
       <c r="AB13">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="AC13">
-        <v>0.91</v>
+        <v>0.94</v>
       </c>
       <c r="AD13">
-        <v>0.93</v>
+        <v>0.99</v>
       </c>
       <c r="AE13">
         <v>0.15</v>
@@ -18942,7 +18942,7 @@
         <v>0.62</v>
       </c>
       <c r="AG13">
-        <v>0.93</v>
+        <v>0.99</v>
       </c>
       <c r="AH13" t="str">
         <v>ĐẠT</v>
@@ -19007,10 +19007,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S14">
-        <v>30.3</v>
+        <v>29.9</v>
       </c>
       <c r="T14">
-        <v>56.3</v>
+        <v>58.3</v>
       </c>
       <c r="U14">
         <v>2.75</v>
@@ -19031,16 +19031,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA14">
-        <v>0.78</v>
+        <v>0.8</v>
       </c>
       <c r="AB14">
         <v>0.67</v>
       </c>
       <c r="AC14">
-        <v>0.94</v>
+        <v>0.97</v>
       </c>
       <c r="AD14">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AE14">
         <v>0.15</v>
@@ -19049,7 +19049,7 @@
         <v>0.62</v>
       </c>
       <c r="AG14">
-        <v>0.94</v>
+        <v>0.98</v>
       </c>
       <c r="AH14" t="str">
         <v>ĐẠT</v>
@@ -19114,40 +19114,40 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S15">
-        <v>28.1</v>
+        <v>27.6</v>
       </c>
       <c r="T15">
-        <v>67.1</v>
+        <v>69.2</v>
       </c>
       <c r="U15">
-        <v>3</v>
+        <v>3.25</v>
       </c>
       <c r="V15">
         <v>0.4</v>
       </c>
       <c r="W15">
-        <v>54</v>
+        <v>63.4</v>
       </c>
       <c r="X15">
-        <v>3.58</v>
+        <v>4.21</v>
       </c>
       <c r="Y15">
-        <v>9.2</v>
+        <v>10.8</v>
       </c>
       <c r="Z15" t="str">
         <v>Ø12 a200</v>
       </c>
       <c r="AA15">
-        <v>0.84</v>
+        <v>0.78</v>
       </c>
       <c r="AB15">
-        <v>0.61</v>
+        <v>0.55</v>
       </c>
       <c r="AC15">
-        <v>0.99</v>
+        <v>0.93</v>
       </c>
       <c r="AD15">
-        <v>0.96</v>
+        <v>0.71</v>
       </c>
       <c r="AE15">
         <v>0.15</v>
@@ -19156,7 +19156,7 @@
         <v>0.62</v>
       </c>
       <c r="AG15">
-        <v>0.99</v>
+        <v>0.93</v>
       </c>
       <c r="AH15" t="str">
         <v>ĐẠT</v>
@@ -19221,10 +19221,10 @@
         <v>B5A-D32 căng, B3A-D36 chùng (MN cao)</v>
       </c>
       <c r="S16">
-        <v>77.9</v>
+        <v>77.5</v>
       </c>
       <c r="T16">
-        <v>29.9</v>
+        <v>31.2</v>
       </c>
       <c r="U16">
         <v>2.75</v>
@@ -19245,16 +19245,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA16">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="AB16">
         <v>0.81</v>
       </c>
       <c r="AC16">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="AD16">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="AE16">
         <v>0.15</v>
@@ -19263,7 +19263,7 @@
         <v>0.62</v>
       </c>
       <c r="AG16">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="AH16" t="str">
         <v>ĐẠT</v>
@@ -19328,10 +19328,10 @@
         <v>B5A-D31 căng, B3A-D37 chùng (MN cao)</v>
       </c>
       <c r="S17">
-        <v>77.9</v>
+        <v>77.5</v>
       </c>
       <c r="T17">
-        <v>29.9</v>
+        <v>31.2</v>
       </c>
       <c r="U17">
         <v>2.75</v>
@@ -19352,16 +19352,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA17">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="AB17">
         <v>0.81</v>
       </c>
       <c r="AC17">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="AD17">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="AE17">
         <v>0.15</v>
@@ -19370,7 +19370,7 @@
         <v>0.62</v>
       </c>
       <c r="AG17">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="AH17" t="str">
         <v>ĐẠT</v>
@@ -19435,10 +19435,10 @@
         <v>B5A-D30 căng, B3A-D38 chùng (MN cao)</v>
       </c>
       <c r="S18">
-        <v>77.9</v>
+        <v>77.5</v>
       </c>
       <c r="T18">
-        <v>30</v>
+        <v>31.3</v>
       </c>
       <c r="U18">
         <v>2.75</v>
@@ -19459,16 +19459,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA18">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="AB18">
         <v>0.81</v>
       </c>
       <c r="AC18">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="AD18">
-        <v>0.68</v>
+        <v>0.72</v>
       </c>
       <c r="AE18">
         <v>0.15</v>
@@ -19477,7 +19477,7 @@
         <v>0.62</v>
       </c>
       <c r="AG18">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="AH18" t="str">
         <v>ĐẠT</v>
@@ -19542,10 +19542,10 @@
         <v>B5A-D29 căng, B3A-D39 chùng (MN cao)</v>
       </c>
       <c r="S19">
-        <v>77.9</v>
+        <v>77.5</v>
       </c>
       <c r="T19">
-        <v>30</v>
+        <v>31.3</v>
       </c>
       <c r="U19">
         <v>2.75</v>
@@ -19566,16 +19566,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA19">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="AB19">
         <v>0.81</v>
       </c>
       <c r="AC19">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="AD19">
-        <v>0.68</v>
+        <v>0.72</v>
       </c>
       <c r="AE19">
         <v>0.15</v>
@@ -19584,7 +19584,7 @@
         <v>0.62</v>
       </c>
       <c r="AG19">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="AH19" t="str">
         <v>ĐẠT</v>
@@ -19649,10 +19649,10 @@
         <v>B5A-D28 căng, B3A-D40 chùng (MN cao)</v>
       </c>
       <c r="S20">
-        <v>77.9</v>
+        <v>77.5</v>
       </c>
       <c r="T20">
-        <v>29.9</v>
+        <v>31.2</v>
       </c>
       <c r="U20">
         <v>2.75</v>
@@ -19673,16 +19673,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA20">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="AB20">
         <v>0.81</v>
       </c>
       <c r="AC20">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="AD20">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="AE20">
         <v>0.15</v>
@@ -19691,7 +19691,7 @@
         <v>0.62</v>
       </c>
       <c r="AG20">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="AH20" t="str">
         <v>ĐẠT</v>
@@ -19756,10 +19756,10 @@
         <v>B5A-D27 căng, B3A-D41 chùng (MN cao)</v>
       </c>
       <c r="S21">
-        <v>77.9</v>
+        <v>77.5</v>
       </c>
       <c r="T21">
-        <v>29.9</v>
+        <v>31.2</v>
       </c>
       <c r="U21">
         <v>2.75</v>
@@ -19780,16 +19780,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA21">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="AB21">
         <v>0.81</v>
       </c>
       <c r="AC21">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="AD21">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="AE21">
         <v>0.15</v>
@@ -19798,7 +19798,7 @@
         <v>0.62</v>
       </c>
       <c r="AG21">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="AH21" t="str">
         <v>ĐẠT</v>
@@ -19863,10 +19863,10 @@
         <v>B5A-D26 căng, B3A-D42 chùng (MN cao)</v>
       </c>
       <c r="S22">
-        <v>77.9</v>
+        <v>77.5</v>
       </c>
       <c r="T22">
-        <v>29.8</v>
+        <v>31.1</v>
       </c>
       <c r="U22">
         <v>2.75</v>
@@ -19887,16 +19887,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA22">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="AB22">
         <v>0.81</v>
       </c>
       <c r="AC22">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="AD22">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="AE22">
         <v>0.15</v>
@@ -19905,7 +19905,7 @@
         <v>0.62</v>
       </c>
       <c r="AG22">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="AH22" t="str">
         <v>ĐẠT</v>
@@ -19970,10 +19970,10 @@
         <v>B5A-D25 căng, B3A-D43 chùng (MN cao)</v>
       </c>
       <c r="S23">
-        <v>77.9</v>
+        <v>77.5</v>
       </c>
       <c r="T23">
-        <v>29.8</v>
+        <v>31.1</v>
       </c>
       <c r="U23">
         <v>2.75</v>
@@ -19994,16 +19994,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA23">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="AB23">
         <v>0.81</v>
       </c>
       <c r="AC23">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="AD23">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="AE23">
         <v>0.15</v>
@@ -20012,7 +20012,7 @@
         <v>0.62</v>
       </c>
       <c r="AG23">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="AH23" t="str">
         <v>ĐẠT</v>
@@ -20077,10 +20077,10 @@
         <v>B5A-D24 căng, B3A-D44 chùng (MN cao)</v>
       </c>
       <c r="S24">
-        <v>77.9</v>
+        <v>77.5</v>
       </c>
       <c r="T24">
-        <v>29.8</v>
+        <v>31.1</v>
       </c>
       <c r="U24">
         <v>2.75</v>
@@ -20101,16 +20101,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA24">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="AB24">
         <v>0.81</v>
       </c>
       <c r="AC24">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="AD24">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="AE24">
         <v>0.15</v>
@@ -20119,7 +20119,7 @@
         <v>0.62</v>
       </c>
       <c r="AG24">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="AH24" t="str">
         <v>ĐẠT</v>
@@ -20184,10 +20184,10 @@
         <v>B5A-D23 căng, B3A-D45 chùng (MN cao)</v>
       </c>
       <c r="S25">
-        <v>77.9</v>
+        <v>77.5</v>
       </c>
       <c r="T25">
-        <v>29.8</v>
+        <v>31.1</v>
       </c>
       <c r="U25">
         <v>2.75</v>
@@ -20208,16 +20208,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA25">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="AB25">
         <v>0.81</v>
       </c>
       <c r="AC25">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="AD25">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="AE25">
         <v>0.15</v>
@@ -20226,7 +20226,7 @@
         <v>0.62</v>
       </c>
       <c r="AG25">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="AH25" t="str">
         <v>ĐẠT</v>
@@ -20291,10 +20291,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S26">
-        <v>25.1</v>
+        <v>24.9</v>
       </c>
       <c r="T26">
-        <v>53.2</v>
+        <v>55.3</v>
       </c>
       <c r="U26">
         <v>2.75</v>
@@ -20315,16 +20315,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA26">
-        <v>0.73</v>
+        <v>0.76</v>
       </c>
       <c r="AB26">
         <v>0.67</v>
       </c>
       <c r="AC26">
-        <v>0.87</v>
+        <v>0.9</v>
       </c>
       <c r="AD26">
-        <v>0.75</v>
+        <v>0.81</v>
       </c>
       <c r="AE26">
         <v>0.15</v>
@@ -20333,7 +20333,7 @@
         <v>0.62</v>
       </c>
       <c r="AG26">
-        <v>0.87</v>
+        <v>0.9</v>
       </c>
       <c r="AH26" t="str">
         <v>ĐẠT</v>
@@ -20398,10 +20398,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S27">
-        <v>25.1</v>
+        <v>24.9</v>
       </c>
       <c r="T27">
-        <v>53.1</v>
+        <v>55.2</v>
       </c>
       <c r="U27">
         <v>2.75</v>
@@ -20422,16 +20422,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA27">
-        <v>0.73</v>
+        <v>0.76</v>
       </c>
       <c r="AB27">
         <v>0.67</v>
       </c>
       <c r="AC27">
-        <v>0.87</v>
+        <v>0.9</v>
       </c>
       <c r="AD27">
-        <v>0.75</v>
+        <v>0.81</v>
       </c>
       <c r="AE27">
         <v>0.15</v>
@@ -20440,7 +20440,7 @@
         <v>0.62</v>
       </c>
       <c r="AG27">
-        <v>0.87</v>
+        <v>0.9</v>
       </c>
       <c r="AH27" t="str">
         <v>ĐẠT</v>
@@ -20505,10 +20505,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S28">
-        <v>25.1</v>
+        <v>24.9</v>
       </c>
       <c r="T28">
-        <v>53.3</v>
+        <v>55.3</v>
       </c>
       <c r="U28">
         <v>2.75</v>
@@ -20529,16 +20529,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA28">
-        <v>0.73</v>
+        <v>0.76</v>
       </c>
       <c r="AB28">
         <v>0.67</v>
       </c>
       <c r="AC28">
-        <v>0.87</v>
+        <v>0.9</v>
       </c>
       <c r="AD28">
-        <v>0.75</v>
+        <v>0.82</v>
       </c>
       <c r="AE28">
         <v>0.15</v>
@@ -20547,7 +20547,7 @@
         <v>0.62</v>
       </c>
       <c r="AG28">
-        <v>0.87</v>
+        <v>0.9</v>
       </c>
       <c r="AH28" t="str">
         <v>ĐẠT</v>
@@ -20612,10 +20612,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S29">
-        <v>25.1</v>
+        <v>24.9</v>
       </c>
       <c r="T29">
-        <v>53.2</v>
+        <v>55.3</v>
       </c>
       <c r="U29">
         <v>2.75</v>
@@ -20636,16 +20636,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA29">
-        <v>0.73</v>
+        <v>0.76</v>
       </c>
       <c r="AB29">
         <v>0.67</v>
       </c>
       <c r="AC29">
-        <v>0.87</v>
+        <v>0.9</v>
       </c>
       <c r="AD29">
-        <v>0.75</v>
+        <v>0.81</v>
       </c>
       <c r="AE29">
         <v>0.15</v>
@@ -20654,7 +20654,7 @@
         <v>0.62</v>
       </c>
       <c r="AG29">
-        <v>0.87</v>
+        <v>0.9</v>
       </c>
       <c r="AH29" t="str">
         <v>ĐẠT</v>
@@ -20719,10 +20719,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S30">
-        <v>25.1</v>
+        <v>24.9</v>
       </c>
       <c r="T30">
-        <v>53.3</v>
+        <v>55.4</v>
       </c>
       <c r="U30">
         <v>2.75</v>
@@ -20743,16 +20743,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA30">
-        <v>0.74</v>
+        <v>0.76</v>
       </c>
       <c r="AB30">
         <v>0.67</v>
       </c>
       <c r="AC30">
-        <v>0.87</v>
+        <v>0.9</v>
       </c>
       <c r="AD30">
-        <v>0.75</v>
+        <v>0.82</v>
       </c>
       <c r="AE30">
         <v>0.15</v>
@@ -20761,7 +20761,7 @@
         <v>0.62</v>
       </c>
       <c r="AG30">
-        <v>0.87</v>
+        <v>0.9</v>
       </c>
       <c r="AH30" t="str">
         <v>ĐẠT</v>
@@ -20826,10 +20826,10 @@
         <v>B5A-D13 căng, B6-D27 chùng (MN cao)</v>
       </c>
       <c r="S31">
-        <v>78.1</v>
+        <v>77.7</v>
       </c>
       <c r="T31">
-        <v>29.4</v>
+        <v>30.7</v>
       </c>
       <c r="U31">
         <v>2.75</v>
@@ -20850,16 +20850,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA31">
-        <v>0.56</v>
+        <v>0.59</v>
       </c>
       <c r="AB31">
         <v>0.81</v>
       </c>
       <c r="AC31">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="AD31">
-        <v>0.66</v>
+        <v>0.7</v>
       </c>
       <c r="AE31">
         <v>0.15</v>
@@ -20868,7 +20868,7 @@
         <v>0.62</v>
       </c>
       <c r="AG31">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="AH31" t="str">
         <v>ĐẠT</v>
@@ -20933,10 +20933,10 @@
         <v>B5A-D14 căng, B6-D31 chùng (MN cao)</v>
       </c>
       <c r="S32">
-        <v>77.2</v>
+        <v>76.7</v>
       </c>
       <c r="T32">
-        <v>32.1</v>
+        <v>33.5</v>
       </c>
       <c r="U32">
         <v>2.75</v>
@@ -20957,16 +20957,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA32">
-        <v>0.61</v>
+        <v>0.64</v>
       </c>
       <c r="AB32">
-        <v>0.81</v>
+        <v>0.85</v>
       </c>
       <c r="AC32">
-        <v>0.87</v>
+        <v>0.89</v>
       </c>
       <c r="AD32">
-        <v>0.74</v>
+        <v>0.78</v>
       </c>
       <c r="AE32">
         <v>0.15</v>
@@ -20975,7 +20975,7 @@
         <v>0.62</v>
       </c>
       <c r="AG32">
-        <v>0.87</v>
+        <v>0.89</v>
       </c>
       <c r="AH32" t="str">
         <v>ĐẠT</v>
@@ -21040,10 +21040,10 @@
         <v>B5A-D15 căng, B6-D17 chùng (MN cao)</v>
       </c>
       <c r="S33">
-        <v>78.1</v>
+        <v>77.7</v>
       </c>
       <c r="T33">
-        <v>29.2</v>
+        <v>30.5</v>
       </c>
       <c r="U33">
         <v>2.75</v>
@@ -21064,16 +21064,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA33">
-        <v>0.56</v>
+        <v>0.58</v>
       </c>
       <c r="AB33">
         <v>0.81</v>
       </c>
       <c r="AC33">
-        <v>0.83</v>
+        <v>0.85</v>
       </c>
       <c r="AD33">
-        <v>0.65</v>
+        <v>0.69</v>
       </c>
       <c r="AE33">
         <v>0.15</v>
@@ -21082,7 +21082,7 @@
         <v>0.62</v>
       </c>
       <c r="AG33">
-        <v>0.83</v>
+        <v>0.85</v>
       </c>
       <c r="AH33" t="str">
         <v>ĐẠT</v>
@@ -21147,10 +21147,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S34">
-        <v>11.5</v>
+        <v>11.4</v>
       </c>
       <c r="T34">
-        <v>55.2</v>
+        <v>57.1</v>
       </c>
       <c r="U34">
         <v>2.5</v>
@@ -21171,16 +21171,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA34">
-        <v>0.84</v>
+        <v>0.87</v>
       </c>
       <c r="AB34">
         <v>0.59</v>
       </c>
       <c r="AC34">
-        <v>0.9</v>
+        <v>0.92</v>
       </c>
       <c r="AD34">
-        <v>0.89</v>
+        <v>0.95</v>
       </c>
       <c r="AE34">
         <v>0.15</v>
@@ -21189,7 +21189,7 @@
         <v>0.62</v>
       </c>
       <c r="AG34">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="AH34" t="str">
         <v>ĐẠT</v>
@@ -21254,10 +21254,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S35">
-        <v>12.1</v>
+        <v>11.9</v>
       </c>
       <c r="T35">
-        <v>47.7</v>
+        <v>49.5</v>
       </c>
       <c r="U35">
         <v>2.5</v>
@@ -21278,16 +21278,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA35">
-        <v>0.73</v>
+        <v>0.76</v>
       </c>
       <c r="AB35">
         <v>0.59</v>
       </c>
       <c r="AC35">
-        <v>0.79</v>
+        <v>0.81</v>
       </c>
       <c r="AD35">
-        <v>0.65</v>
+        <v>0.71</v>
       </c>
       <c r="AE35">
         <v>0.15</v>
@@ -21296,7 +21296,7 @@
         <v>0.62</v>
       </c>
       <c r="AG35">
-        <v>0.79</v>
+        <v>0.81</v>
       </c>
       <c r="AH35" t="str">
         <v>ĐẠT</v>
@@ -21361,10 +21361,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S36">
-        <v>11.6</v>
+        <v>11.4</v>
       </c>
       <c r="T36">
-        <v>54.4</v>
+        <v>56.3</v>
       </c>
       <c r="U36">
         <v>2.5</v>
@@ -21385,16 +21385,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA36">
-        <v>0.83</v>
+        <v>0.86</v>
       </c>
       <c r="AB36">
         <v>0.59</v>
       </c>
       <c r="AC36">
-        <v>0.89</v>
+        <v>0.91</v>
       </c>
       <c r="AD36">
-        <v>0.87</v>
+        <v>0.93</v>
       </c>
       <c r="AE36">
         <v>0.15</v>
@@ -21403,7 +21403,7 @@
         <v>0.62</v>
       </c>
       <c r="AG36">
-        <v>0.89</v>
+        <v>0.93</v>
       </c>
       <c r="AH36" t="str">
         <v>ĐẠT</v>
@@ -21468,10 +21468,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S37">
-        <v>11.5</v>
+        <v>11.3</v>
       </c>
       <c r="T37">
-        <v>56</v>
+        <v>57.9</v>
       </c>
       <c r="U37">
         <v>2.5</v>
@@ -21492,16 +21492,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA37">
-        <v>0.86</v>
+        <v>0.89</v>
       </c>
       <c r="AB37">
-        <v>0.59</v>
+        <v>0.58</v>
       </c>
       <c r="AC37">
-        <v>0.91</v>
+        <v>0.94</v>
       </c>
       <c r="AD37">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AE37">
         <v>0.15</v>
@@ -21510,7 +21510,7 @@
         <v>0.62</v>
       </c>
       <c r="AG37">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AH37" t="str">
         <v>ĐẠT</v>
@@ -21575,10 +21575,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S38">
-        <v>24</v>
+        <v>23.7</v>
       </c>
       <c r="T38">
-        <v>47.6</v>
+        <v>49.2</v>
       </c>
       <c r="U38">
         <v>2.5</v>
@@ -21599,16 +21599,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA38">
-        <v>0.73</v>
+        <v>0.75</v>
       </c>
       <c r="AB38">
         <v>0.59</v>
       </c>
       <c r="AC38">
-        <v>0.86</v>
+        <v>0.89</v>
       </c>
       <c r="AD38">
-        <v>0.82</v>
+        <v>0.87</v>
       </c>
       <c r="AE38">
         <v>0.15</v>
@@ -21617,7 +21617,7 @@
         <v>0.62</v>
       </c>
       <c r="AG38">
-        <v>0.86</v>
+        <v>0.89</v>
       </c>
       <c r="AH38" t="str">
         <v>ĐẠT</v>
@@ -21685,7 +21685,7 @@
         <v>Bê tông đế</v>
       </c>
       <c r="B45">
-        <v>92.2</v>
+        <v>92.8</v>
       </c>
       <c r="C45" t="str">
         <v>m³</v>
@@ -21726,10 +21726,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Số đế cạnh B = 3,00 m</v>
+        <v>Số đế cạnh B = 3,25 m</v>
       </c>
       <c r="B49">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C49" t="str">
         <v>đế</v>
@@ -21737,29 +21737,18 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Số đế cạnh B = 3,25 m</v>
+        <v>Số đế mà địa hình IFC cao hơn đáy thiết kế trên 0,5 m (cần kiểm tra khảo sát / nạo vét)</v>
       </c>
       <c r="B50">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C50" t="str">
         <v>đế</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="str">
-        <v>Số đế mà địa hình IFC cao hơn đáy thiết kế trên 0,5 m (cần kiểm tra khảo sát / nạo vét)</v>
-      </c>
-      <c r="B51">
-        <v>4</v>
-      </c>
-      <c r="C51" t="str">
-        <v>đế</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AI51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AI50"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>